<commit_message>
Figure 3F: add cumulative-burden sheet
A grouped bar of seizure burden hides the structure: the SV2A group is bimodal
— 4 animals at exactly 0 for all 21 baseline days, 2 non-responders as high as
EGFP — so mean +/- SEM overlaps (225 +/- 78 vs 45 +/- 29 min) while the medians
are 87.7 vs 0.8 min.

Sheet 3 gives cumulative seizure minutes per animal per baseline day as an XY
table: every animal a thin grey line, group medians bold. Zeros become flat
lines along the axis, which reads as "never seized" rather than a plotting
floor, and the two non-responders are visible rather than averaged away.
Notes specify testing the day-21 endpoint by Mann-Whitney (p = 0.0032) rather
than a 2-way ANOVA over days, since cumulative values are not independent.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Figure3_replacement_panels.xlsx
+++ b/Figure3_replacement_panels.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1_TimeToFirstSeizure_KM" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2_SeizureBurden" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3_CumulativeBurden" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1254,4 +1255,1807 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:W49"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="11" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
+    <col width="12" customWidth="1" min="14" max="14"/>
+    <col width="12" customWidth="1" min="15" max="15"/>
+    <col width="12" customWidth="1" min="16" max="16"/>
+    <col width="12" customWidth="1" min="17" max="17"/>
+    <col width="12" customWidth="1" min="18" max="18"/>
+    <col width="12" customWidth="1" min="19" max="19"/>
+    <col width="12" customWidth="1" min="20" max="20"/>
+    <col width="12" customWidth="1" min="21" max="21"/>
+    <col width="12" customWidth="1" min="22" max="22"/>
+    <col width="12" customWidth="1" min="23" max="23"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Cumulative seizure time (minutes) over baseline days 1-21, confidence &gt;= 0.5</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>PRISM TABLE TYPE:  XY, with X = day and one Y column per animal (Y = single values, no replicates)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Plot every animal as a thin grey line; overlay the two group MEDIAN columns as bold lines. Do not use mean +/- SEM — see note.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>X  (day)</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>EGFP 25</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>EGFP 31</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>EGFP 33</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>EGFP 355675</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>EGFP 355679</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>EGFP 372833</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>EGFP 372838</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>SV2A 24</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>SV2A 26</t>
+        </is>
+      </c>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>SV2A 29</t>
+        </is>
+      </c>
+      <c r="L6" s="2" t="inlineStr">
+        <is>
+          <t>SV2A 32</t>
+        </is>
+      </c>
+      <c r="M6" s="2" t="inlineStr">
+        <is>
+          <t>SV2A 355668</t>
+        </is>
+      </c>
+      <c r="N6" s="2" t="inlineStr">
+        <is>
+          <t>SV2A 355669</t>
+        </is>
+      </c>
+      <c r="O6" s="2" t="inlineStr">
+        <is>
+          <t>SV2A 355670</t>
+        </is>
+      </c>
+      <c r="P6" s="2" t="inlineStr">
+        <is>
+          <t>SV2A 355673</t>
+        </is>
+      </c>
+      <c r="Q6" s="2" t="inlineStr">
+        <is>
+          <t>SV2A 355677</t>
+        </is>
+      </c>
+      <c r="R6" s="2" t="inlineStr">
+        <is>
+          <t>SV2A 372828</t>
+        </is>
+      </c>
+      <c r="S6" s="2" t="inlineStr">
+        <is>
+          <t>SV2A 372829</t>
+        </is>
+      </c>
+      <c r="T6" s="2" t="inlineStr">
+        <is>
+          <t>SV2A 372830</t>
+        </is>
+      </c>
+      <c r="U6" s="2" t="inlineStr">
+        <is>
+          <t>SV2A 372832</t>
+        </is>
+      </c>
+      <c r="V6" s="2" t="inlineStr">
+        <is>
+          <t>EGFP median</t>
+        </is>
+      </c>
+      <c r="W6" s="2" t="inlineStr">
+        <is>
+          <t>SV2A median</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>1</v>
+      </c>
+      <c r="B7" t="n">
+        <v>3.777</v>
+      </c>
+      <c r="C7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" t="n">
+        <v>8.137</v>
+      </c>
+      <c r="F7" t="n">
+        <v>4.501</v>
+      </c>
+      <c r="G7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J7" t="n">
+        <v>1.174</v>
+      </c>
+      <c r="K7" t="n">
+        <v>17.018</v>
+      </c>
+      <c r="L7" t="n">
+        <v>2.981</v>
+      </c>
+      <c r="M7" t="n">
+        <v>0</v>
+      </c>
+      <c r="N7" t="n">
+        <v>0</v>
+      </c>
+      <c r="O7" t="n">
+        <v>0</v>
+      </c>
+      <c r="P7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q7" t="n">
+        <v>0</v>
+      </c>
+      <c r="R7" t="n">
+        <v>0</v>
+      </c>
+      <c r="S7" t="n">
+        <v>0</v>
+      </c>
+      <c r="T7" t="n">
+        <v>0</v>
+      </c>
+      <c r="U7" t="n">
+        <v>0</v>
+      </c>
+      <c r="V7" t="n">
+        <v>0</v>
+      </c>
+      <c r="W7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>2</v>
+      </c>
+      <c r="B8" t="n">
+        <v>5.25</v>
+      </c>
+      <c r="C8" t="n">
+        <v>0</v>
+      </c>
+      <c r="D8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" t="n">
+        <v>23.419</v>
+      </c>
+      <c r="F8" t="n">
+        <v>7.226</v>
+      </c>
+      <c r="G8" t="n">
+        <v>1.865</v>
+      </c>
+      <c r="H8" t="n">
+        <v>8.156000000000001</v>
+      </c>
+      <c r="I8" t="n">
+        <v>0</v>
+      </c>
+      <c r="J8" t="n">
+        <v>1.278</v>
+      </c>
+      <c r="K8" t="n">
+        <v>22.114</v>
+      </c>
+      <c r="L8" t="n">
+        <v>5.109</v>
+      </c>
+      <c r="M8" t="n">
+        <v>0</v>
+      </c>
+      <c r="N8" t="n">
+        <v>0</v>
+      </c>
+      <c r="O8" t="n">
+        <v>0</v>
+      </c>
+      <c r="P8" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q8" t="n">
+        <v>0</v>
+      </c>
+      <c r="R8" t="n">
+        <v>0</v>
+      </c>
+      <c r="S8" t="n">
+        <v>0</v>
+      </c>
+      <c r="T8" t="n">
+        <v>0</v>
+      </c>
+      <c r="U8" t="n">
+        <v>0</v>
+      </c>
+      <c r="V8" t="n">
+        <v>5.25</v>
+      </c>
+      <c r="W8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>3</v>
+      </c>
+      <c r="B9" t="n">
+        <v>6.235</v>
+      </c>
+      <c r="C9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" t="n">
+        <v>41.704</v>
+      </c>
+      <c r="F9" t="n">
+        <v>11.329</v>
+      </c>
+      <c r="G9" t="n">
+        <v>3.768</v>
+      </c>
+      <c r="H9" t="n">
+        <v>10.328</v>
+      </c>
+      <c r="I9" t="n">
+        <v>0</v>
+      </c>
+      <c r="J9" t="n">
+        <v>1.278</v>
+      </c>
+      <c r="K9" t="n">
+        <v>30.063</v>
+      </c>
+      <c r="L9" t="n">
+        <v>9.436999999999999</v>
+      </c>
+      <c r="M9" t="n">
+        <v>0</v>
+      </c>
+      <c r="N9" t="n">
+        <v>0.261</v>
+      </c>
+      <c r="O9" t="n">
+        <v>0</v>
+      </c>
+      <c r="P9" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q9" t="n">
+        <v>0</v>
+      </c>
+      <c r="R9" t="n">
+        <v>0</v>
+      </c>
+      <c r="S9" t="n">
+        <v>0.436</v>
+      </c>
+      <c r="T9" t="n">
+        <v>0.626</v>
+      </c>
+      <c r="U9" t="n">
+        <v>0</v>
+      </c>
+      <c r="V9" t="n">
+        <v>6.235</v>
+      </c>
+      <c r="W9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>4</v>
+      </c>
+      <c r="B10" t="n">
+        <v>9.663</v>
+      </c>
+      <c r="C10" t="n">
+        <v>2.561</v>
+      </c>
+      <c r="D10" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" t="n">
+        <v>61.922</v>
+      </c>
+      <c r="F10" t="n">
+        <v>18.563</v>
+      </c>
+      <c r="G10" t="n">
+        <v>6.413</v>
+      </c>
+      <c r="H10" t="n">
+        <v>13.633</v>
+      </c>
+      <c r="I10" t="n">
+        <v>1.317</v>
+      </c>
+      <c r="J10" t="n">
+        <v>1.598</v>
+      </c>
+      <c r="K10" t="n">
+        <v>37.563</v>
+      </c>
+      <c r="L10" t="n">
+        <v>18.395</v>
+      </c>
+      <c r="M10" t="n">
+        <v>0</v>
+      </c>
+      <c r="N10" t="n">
+        <v>0.261</v>
+      </c>
+      <c r="O10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P10" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q10" t="n">
+        <v>0</v>
+      </c>
+      <c r="R10" t="n">
+        <v>0</v>
+      </c>
+      <c r="S10" t="n">
+        <v>0.645</v>
+      </c>
+      <c r="T10" t="n">
+        <v>0.626</v>
+      </c>
+      <c r="U10" t="n">
+        <v>0</v>
+      </c>
+      <c r="V10" t="n">
+        <v>9.663</v>
+      </c>
+      <c r="W10" t="n">
+        <v>0.261</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>5</v>
+      </c>
+      <c r="B11" t="n">
+        <v>13.277</v>
+      </c>
+      <c r="C11" t="n">
+        <v>3.493</v>
+      </c>
+      <c r="D11" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" t="n">
+        <v>107.61</v>
+      </c>
+      <c r="F11" t="n">
+        <v>30.952</v>
+      </c>
+      <c r="G11" t="n">
+        <v>10.624</v>
+      </c>
+      <c r="H11" t="n">
+        <v>31.862</v>
+      </c>
+      <c r="I11" t="n">
+        <v>1.317</v>
+      </c>
+      <c r="J11" t="n">
+        <v>1.598</v>
+      </c>
+      <c r="K11" t="n">
+        <v>40.302</v>
+      </c>
+      <c r="L11" t="n">
+        <v>25.484</v>
+      </c>
+      <c r="M11" t="n">
+        <v>0</v>
+      </c>
+      <c r="N11" t="n">
+        <v>0.779</v>
+      </c>
+      <c r="O11" t="n">
+        <v>0</v>
+      </c>
+      <c r="P11" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q11" t="n">
+        <v>0</v>
+      </c>
+      <c r="R11" t="n">
+        <v>0</v>
+      </c>
+      <c r="S11" t="n">
+        <v>0.645</v>
+      </c>
+      <c r="T11" t="n">
+        <v>0.626</v>
+      </c>
+      <c r="U11" t="n">
+        <v>0</v>
+      </c>
+      <c r="V11" t="n">
+        <v>13.277</v>
+      </c>
+      <c r="W11" t="n">
+        <v>0.626</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>6</v>
+      </c>
+      <c r="B12" t="n">
+        <v>18.357</v>
+      </c>
+      <c r="C12" t="n">
+        <v>6.629</v>
+      </c>
+      <c r="D12" t="n">
+        <v>0</v>
+      </c>
+      <c r="E12" t="n">
+        <v>107.61</v>
+      </c>
+      <c r="F12" t="n">
+        <v>30.952</v>
+      </c>
+      <c r="G12" t="n">
+        <v>10.624</v>
+      </c>
+      <c r="H12" t="n">
+        <v>31.862</v>
+      </c>
+      <c r="I12" t="n">
+        <v>1.317</v>
+      </c>
+      <c r="J12" t="n">
+        <v>1.598</v>
+      </c>
+      <c r="K12" t="n">
+        <v>45.075</v>
+      </c>
+      <c r="L12" t="n">
+        <v>45.433</v>
+      </c>
+      <c r="M12" t="n">
+        <v>0</v>
+      </c>
+      <c r="N12" t="n">
+        <v>0.779</v>
+      </c>
+      <c r="O12" t="n">
+        <v>0</v>
+      </c>
+      <c r="P12" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q12" t="n">
+        <v>0</v>
+      </c>
+      <c r="R12" t="n">
+        <v>0</v>
+      </c>
+      <c r="S12" t="n">
+        <v>0.645</v>
+      </c>
+      <c r="T12" t="n">
+        <v>0.626</v>
+      </c>
+      <c r="U12" t="n">
+        <v>0</v>
+      </c>
+      <c r="V12" t="n">
+        <v>18.357</v>
+      </c>
+      <c r="W12" t="n">
+        <v>0.626</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>7</v>
+      </c>
+      <c r="B13" t="n">
+        <v>22.407</v>
+      </c>
+      <c r="C13" t="n">
+        <v>9.331</v>
+      </c>
+      <c r="D13" t="n">
+        <v>0</v>
+      </c>
+      <c r="E13" t="n">
+        <v>126.484</v>
+      </c>
+      <c r="F13" t="n">
+        <v>33.083</v>
+      </c>
+      <c r="G13" t="n">
+        <v>14.536</v>
+      </c>
+      <c r="H13" t="n">
+        <v>36.628</v>
+      </c>
+      <c r="I13" t="n">
+        <v>1.317</v>
+      </c>
+      <c r="J13" t="n">
+        <v>1.598</v>
+      </c>
+      <c r="K13" t="n">
+        <v>67.09999999999999</v>
+      </c>
+      <c r="L13" t="n">
+        <v>63.464</v>
+      </c>
+      <c r="M13" t="n">
+        <v>0</v>
+      </c>
+      <c r="N13" t="n">
+        <v>0.779</v>
+      </c>
+      <c r="O13" t="n">
+        <v>0</v>
+      </c>
+      <c r="P13" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q13" t="n">
+        <v>0</v>
+      </c>
+      <c r="R13" t="n">
+        <v>0</v>
+      </c>
+      <c r="S13" t="n">
+        <v>0.645</v>
+      </c>
+      <c r="T13" t="n">
+        <v>1.276</v>
+      </c>
+      <c r="U13" t="n">
+        <v>0</v>
+      </c>
+      <c r="V13" t="n">
+        <v>22.407</v>
+      </c>
+      <c r="W13" t="n">
+        <v>0.645</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>8</v>
+      </c>
+      <c r="B14" t="n">
+        <v>28.332</v>
+      </c>
+      <c r="C14" t="n">
+        <v>13.248</v>
+      </c>
+      <c r="D14" t="n">
+        <v>0</v>
+      </c>
+      <c r="E14" t="n">
+        <v>158.689</v>
+      </c>
+      <c r="F14" t="n">
+        <v>40.131</v>
+      </c>
+      <c r="G14" t="n">
+        <v>18.88</v>
+      </c>
+      <c r="H14" t="n">
+        <v>36.628</v>
+      </c>
+      <c r="I14" t="n">
+        <v>1.317</v>
+      </c>
+      <c r="J14" t="n">
+        <v>1.598</v>
+      </c>
+      <c r="K14" t="n">
+        <v>111.623</v>
+      </c>
+      <c r="L14" t="n">
+        <v>81.935</v>
+      </c>
+      <c r="M14" t="n">
+        <v>0</v>
+      </c>
+      <c r="N14" t="n">
+        <v>0.889</v>
+      </c>
+      <c r="O14" t="n">
+        <v>0</v>
+      </c>
+      <c r="P14" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q14" t="n">
+        <v>0</v>
+      </c>
+      <c r="R14" t="n">
+        <v>0</v>
+      </c>
+      <c r="S14" t="n">
+        <v>0.645</v>
+      </c>
+      <c r="T14" t="n">
+        <v>2.044</v>
+      </c>
+      <c r="U14" t="n">
+        <v>0</v>
+      </c>
+      <c r="V14" t="n">
+        <v>28.332</v>
+      </c>
+      <c r="W14" t="n">
+        <v>0.645</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>9</v>
+      </c>
+      <c r="B15" t="n">
+        <v>33.647</v>
+      </c>
+      <c r="C15" t="n">
+        <v>18.568</v>
+      </c>
+      <c r="D15" t="n">
+        <v>0.256</v>
+      </c>
+      <c r="E15" t="n">
+        <v>194.037</v>
+      </c>
+      <c r="F15" t="n">
+        <v>44.558</v>
+      </c>
+      <c r="G15" t="n">
+        <v>20.52</v>
+      </c>
+      <c r="H15" t="n">
+        <v>37.625</v>
+      </c>
+      <c r="I15" t="n">
+        <v>1.317</v>
+      </c>
+      <c r="J15" t="n">
+        <v>1.598</v>
+      </c>
+      <c r="K15" t="n">
+        <v>144.082</v>
+      </c>
+      <c r="L15" t="n">
+        <v>103.187</v>
+      </c>
+      <c r="M15" t="n">
+        <v>0</v>
+      </c>
+      <c r="N15" t="n">
+        <v>0.889</v>
+      </c>
+      <c r="O15" t="n">
+        <v>0</v>
+      </c>
+      <c r="P15" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q15" t="n">
+        <v>0</v>
+      </c>
+      <c r="R15" t="n">
+        <v>0</v>
+      </c>
+      <c r="S15" t="n">
+        <v>0.645</v>
+      </c>
+      <c r="T15" t="n">
+        <v>2.044</v>
+      </c>
+      <c r="U15" t="n">
+        <v>0</v>
+      </c>
+      <c r="V15" t="n">
+        <v>33.647</v>
+      </c>
+      <c r="W15" t="n">
+        <v>0.645</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>10</v>
+      </c>
+      <c r="B16" t="n">
+        <v>42.312</v>
+      </c>
+      <c r="C16" t="n">
+        <v>24.996</v>
+      </c>
+      <c r="D16" t="n">
+        <v>0.756</v>
+      </c>
+      <c r="E16" t="n">
+        <v>251.443</v>
+      </c>
+      <c r="F16" t="n">
+        <v>46.512</v>
+      </c>
+      <c r="G16" t="n">
+        <v>22.846</v>
+      </c>
+      <c r="H16" t="n">
+        <v>46.251</v>
+      </c>
+      <c r="I16" t="n">
+        <v>2.835</v>
+      </c>
+      <c r="J16" t="n">
+        <v>1.598</v>
+      </c>
+      <c r="K16" t="n">
+        <v>160.912</v>
+      </c>
+      <c r="L16" t="n">
+        <v>119.698</v>
+      </c>
+      <c r="M16" t="n">
+        <v>0</v>
+      </c>
+      <c r="N16" t="n">
+        <v>1.704</v>
+      </c>
+      <c r="O16" t="n">
+        <v>0</v>
+      </c>
+      <c r="P16" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q16" t="n">
+        <v>0</v>
+      </c>
+      <c r="R16" t="n">
+        <v>0</v>
+      </c>
+      <c r="S16" t="n">
+        <v>0.645</v>
+      </c>
+      <c r="T16" t="n">
+        <v>2.488</v>
+      </c>
+      <c r="U16" t="n">
+        <v>0</v>
+      </c>
+      <c r="V16" t="n">
+        <v>42.312</v>
+      </c>
+      <c r="W16" t="n">
+        <v>0.645</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>11</v>
+      </c>
+      <c r="B17" t="n">
+        <v>60.44</v>
+      </c>
+      <c r="C17" t="n">
+        <v>35.622</v>
+      </c>
+      <c r="D17" t="n">
+        <v>4.661</v>
+      </c>
+      <c r="E17" t="n">
+        <v>251.443</v>
+      </c>
+      <c r="F17" t="n">
+        <v>46.512</v>
+      </c>
+      <c r="G17" t="n">
+        <v>27.772</v>
+      </c>
+      <c r="H17" t="n">
+        <v>51.071</v>
+      </c>
+      <c r="I17" t="n">
+        <v>3.798</v>
+      </c>
+      <c r="J17" t="n">
+        <v>3.046</v>
+      </c>
+      <c r="K17" t="n">
+        <v>189.689</v>
+      </c>
+      <c r="L17" t="n">
+        <v>151.666</v>
+      </c>
+      <c r="M17" t="n">
+        <v>0</v>
+      </c>
+      <c r="N17" t="n">
+        <v>1.704</v>
+      </c>
+      <c r="O17" t="n">
+        <v>0</v>
+      </c>
+      <c r="P17" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q17" t="n">
+        <v>0</v>
+      </c>
+      <c r="R17" t="n">
+        <v>0</v>
+      </c>
+      <c r="S17" t="n">
+        <v>0.645</v>
+      </c>
+      <c r="T17" t="n">
+        <v>2.488</v>
+      </c>
+      <c r="U17" t="n">
+        <v>0</v>
+      </c>
+      <c r="V17" t="n">
+        <v>46.512</v>
+      </c>
+      <c r="W17" t="n">
+        <v>0.645</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>12</v>
+      </c>
+      <c r="B18" t="n">
+        <v>67.619</v>
+      </c>
+      <c r="C18" t="n">
+        <v>40.11</v>
+      </c>
+      <c r="D18" t="n">
+        <v>9.643000000000001</v>
+      </c>
+      <c r="E18" t="n">
+        <v>280.865</v>
+      </c>
+      <c r="F18" t="n">
+        <v>52.65</v>
+      </c>
+      <c r="G18" t="n">
+        <v>37.209</v>
+      </c>
+      <c r="H18" t="n">
+        <v>58.696</v>
+      </c>
+      <c r="I18" t="n">
+        <v>4.46</v>
+      </c>
+      <c r="J18" t="n">
+        <v>3.666</v>
+      </c>
+      <c r="K18" t="n">
+        <v>212.859</v>
+      </c>
+      <c r="L18" t="n">
+        <v>168.506</v>
+      </c>
+      <c r="M18" t="n">
+        <v>0</v>
+      </c>
+      <c r="N18" t="n">
+        <v>1.704</v>
+      </c>
+      <c r="O18" t="n">
+        <v>0</v>
+      </c>
+      <c r="P18" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q18" t="n">
+        <v>0</v>
+      </c>
+      <c r="R18" t="n">
+        <v>0</v>
+      </c>
+      <c r="S18" t="n">
+        <v>0.645</v>
+      </c>
+      <c r="T18" t="n">
+        <v>3.557</v>
+      </c>
+      <c r="U18" t="n">
+        <v>0</v>
+      </c>
+      <c r="V18" t="n">
+        <v>52.65</v>
+      </c>
+      <c r="W18" t="n">
+        <v>0.645</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>13</v>
+      </c>
+      <c r="B19" t="n">
+        <v>80.44799999999999</v>
+      </c>
+      <c r="C19" t="n">
+        <v>46.453</v>
+      </c>
+      <c r="D19" t="n">
+        <v>16.988</v>
+      </c>
+      <c r="E19" t="n">
+        <v>323.538</v>
+      </c>
+      <c r="F19" t="n">
+        <v>57.78</v>
+      </c>
+      <c r="G19" t="n">
+        <v>37.209</v>
+      </c>
+      <c r="H19" t="n">
+        <v>58.696</v>
+      </c>
+      <c r="I19" t="n">
+        <v>4.46</v>
+      </c>
+      <c r="J19" t="n">
+        <v>3.666</v>
+      </c>
+      <c r="K19" t="n">
+        <v>230.531</v>
+      </c>
+      <c r="L19" t="n">
+        <v>187.336</v>
+      </c>
+      <c r="M19" t="n">
+        <v>0</v>
+      </c>
+      <c r="N19" t="n">
+        <v>2.314</v>
+      </c>
+      <c r="O19" t="n">
+        <v>0</v>
+      </c>
+      <c r="P19" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q19" t="n">
+        <v>0</v>
+      </c>
+      <c r="R19" t="n">
+        <v>0</v>
+      </c>
+      <c r="S19" t="n">
+        <v>0.645</v>
+      </c>
+      <c r="T19" t="n">
+        <v>3.557</v>
+      </c>
+      <c r="U19" t="n">
+        <v>0</v>
+      </c>
+      <c r="V19" t="n">
+        <v>57.78</v>
+      </c>
+      <c r="W19" t="n">
+        <v>0.645</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>14</v>
+      </c>
+      <c r="B20" t="n">
+        <v>90.556</v>
+      </c>
+      <c r="C20" t="n">
+        <v>52.48</v>
+      </c>
+      <c r="D20" t="n">
+        <v>22.657</v>
+      </c>
+      <c r="E20" t="n">
+        <v>323.538</v>
+      </c>
+      <c r="F20" t="n">
+        <v>57.78</v>
+      </c>
+      <c r="G20" t="n">
+        <v>40.414</v>
+      </c>
+      <c r="H20" t="n">
+        <v>61.623</v>
+      </c>
+      <c r="I20" t="n">
+        <v>4.46</v>
+      </c>
+      <c r="J20" t="n">
+        <v>3.666</v>
+      </c>
+      <c r="K20" t="n">
+        <v>269.418</v>
+      </c>
+      <c r="L20" t="n">
+        <v>201.509</v>
+      </c>
+      <c r="M20" t="n">
+        <v>0</v>
+      </c>
+      <c r="N20" t="n">
+        <v>2.314</v>
+      </c>
+      <c r="O20" t="n">
+        <v>0</v>
+      </c>
+      <c r="P20" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q20" t="n">
+        <v>0</v>
+      </c>
+      <c r="R20" t="n">
+        <v>0</v>
+      </c>
+      <c r="S20" t="n">
+        <v>0.645</v>
+      </c>
+      <c r="T20" t="n">
+        <v>3.557</v>
+      </c>
+      <c r="U20" t="n">
+        <v>0</v>
+      </c>
+      <c r="V20" t="n">
+        <v>57.78</v>
+      </c>
+      <c r="W20" t="n">
+        <v>0.645</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>15</v>
+      </c>
+      <c r="B21" t="n">
+        <v>123.142</v>
+      </c>
+      <c r="C21" t="n">
+        <v>65.702</v>
+      </c>
+      <c r="D21" t="n">
+        <v>31.719</v>
+      </c>
+      <c r="E21" t="n">
+        <v>351.599</v>
+      </c>
+      <c r="F21" t="n">
+        <v>60.956</v>
+      </c>
+      <c r="G21" t="n">
+        <v>44.871</v>
+      </c>
+      <c r="H21" t="n">
+        <v>64.04600000000001</v>
+      </c>
+      <c r="I21" t="n">
+        <v>4.46</v>
+      </c>
+      <c r="J21" t="n">
+        <v>3.666</v>
+      </c>
+      <c r="K21" t="n">
+        <v>274.214</v>
+      </c>
+      <c r="L21" t="n">
+        <v>226.165</v>
+      </c>
+      <c r="M21" t="n">
+        <v>0</v>
+      </c>
+      <c r="N21" t="n">
+        <v>2.314</v>
+      </c>
+      <c r="O21" t="n">
+        <v>0</v>
+      </c>
+      <c r="P21" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q21" t="n">
+        <v>0</v>
+      </c>
+      <c r="R21" t="n">
+        <v>0</v>
+      </c>
+      <c r="S21" t="n">
+        <v>0.645</v>
+      </c>
+      <c r="T21" t="n">
+        <v>3.557</v>
+      </c>
+      <c r="U21" t="n">
+        <v>0</v>
+      </c>
+      <c r="V21" t="n">
+        <v>64.04600000000001</v>
+      </c>
+      <c r="W21" t="n">
+        <v>0.645</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>16</v>
+      </c>
+      <c r="B22" t="n">
+        <v>193.203</v>
+      </c>
+      <c r="C22" t="n">
+        <v>72.986</v>
+      </c>
+      <c r="D22" t="n">
+        <v>38.706</v>
+      </c>
+      <c r="E22" t="n">
+        <v>392.31</v>
+      </c>
+      <c r="F22" t="n">
+        <v>62.511</v>
+      </c>
+      <c r="G22" t="n">
+        <v>47.128</v>
+      </c>
+      <c r="H22" t="n">
+        <v>67.16800000000001</v>
+      </c>
+      <c r="I22" t="n">
+        <v>4.46</v>
+      </c>
+      <c r="J22" t="n">
+        <v>3.666</v>
+      </c>
+      <c r="K22" t="n">
+        <v>281.802</v>
+      </c>
+      <c r="L22" t="n">
+        <v>232.404</v>
+      </c>
+      <c r="M22" t="n">
+        <v>0</v>
+      </c>
+      <c r="N22" t="n">
+        <v>2.314</v>
+      </c>
+      <c r="O22" t="n">
+        <v>0</v>
+      </c>
+      <c r="P22" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q22" t="n">
+        <v>0</v>
+      </c>
+      <c r="R22" t="n">
+        <v>0</v>
+      </c>
+      <c r="S22" t="n">
+        <v>0.645</v>
+      </c>
+      <c r="T22" t="n">
+        <v>4.415</v>
+      </c>
+      <c r="U22" t="n">
+        <v>0.539</v>
+      </c>
+      <c r="V22" t="n">
+        <v>67.16800000000001</v>
+      </c>
+      <c r="W22" t="n">
+        <v>0.645</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>17</v>
+      </c>
+      <c r="B23" t="n">
+        <v>245.679</v>
+      </c>
+      <c r="C23" t="n">
+        <v>85.22499999999999</v>
+      </c>
+      <c r="D23" t="n">
+        <v>45.181</v>
+      </c>
+      <c r="E23" t="n">
+        <v>435.401</v>
+      </c>
+      <c r="F23" t="n">
+        <v>65.43600000000001</v>
+      </c>
+      <c r="G23" t="n">
+        <v>48.834</v>
+      </c>
+      <c r="H23" t="n">
+        <v>70.408</v>
+      </c>
+      <c r="I23" t="n">
+        <v>4.46</v>
+      </c>
+      <c r="J23" t="n">
+        <v>3.666</v>
+      </c>
+      <c r="K23" t="n">
+        <v>299.691</v>
+      </c>
+      <c r="L23" t="n">
+        <v>252.786</v>
+      </c>
+      <c r="M23" t="n">
+        <v>0</v>
+      </c>
+      <c r="N23" t="n">
+        <v>2.314</v>
+      </c>
+      <c r="O23" t="n">
+        <v>0</v>
+      </c>
+      <c r="P23" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q23" t="n">
+        <v>0</v>
+      </c>
+      <c r="R23" t="n">
+        <v>0</v>
+      </c>
+      <c r="S23" t="n">
+        <v>0.645</v>
+      </c>
+      <c r="T23" t="n">
+        <v>5.465</v>
+      </c>
+      <c r="U23" t="n">
+        <v>0.539</v>
+      </c>
+      <c r="V23" t="n">
+        <v>70.408</v>
+      </c>
+      <c r="W23" t="n">
+        <v>0.645</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>18</v>
+      </c>
+      <c r="B24" t="n">
+        <v>334.378</v>
+      </c>
+      <c r="C24" t="n">
+        <v>168.448</v>
+      </c>
+      <c r="D24" t="n">
+        <v>45.878</v>
+      </c>
+      <c r="E24" t="n">
+        <v>481.811</v>
+      </c>
+      <c r="F24" t="n">
+        <v>69.66800000000001</v>
+      </c>
+      <c r="G24" t="n">
+        <v>50.579</v>
+      </c>
+      <c r="H24" t="n">
+        <v>74.67</v>
+      </c>
+      <c r="I24" t="n">
+        <v>4.46</v>
+      </c>
+      <c r="J24" t="n">
+        <v>3.666</v>
+      </c>
+      <c r="K24" t="n">
+        <v>300.299</v>
+      </c>
+      <c r="L24" t="n">
+        <v>259.246</v>
+      </c>
+      <c r="M24" t="n">
+        <v>0</v>
+      </c>
+      <c r="N24" t="n">
+        <v>3.226</v>
+      </c>
+      <c r="O24" t="n">
+        <v>0</v>
+      </c>
+      <c r="P24" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q24" t="n">
+        <v>0</v>
+      </c>
+      <c r="R24" t="n">
+        <v>0</v>
+      </c>
+      <c r="S24" t="n">
+        <v>0.645</v>
+      </c>
+      <c r="T24" t="n">
+        <v>5.465</v>
+      </c>
+      <c r="U24" t="n">
+        <v>0.539</v>
+      </c>
+      <c r="V24" t="n">
+        <v>74.67</v>
+      </c>
+      <c r="W24" t="n">
+        <v>0.645</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>19</v>
+      </c>
+      <c r="B25" t="n">
+        <v>334.378</v>
+      </c>
+      <c r="C25" t="n">
+        <v>168.448</v>
+      </c>
+      <c r="D25" t="n">
+        <v>45.878</v>
+      </c>
+      <c r="E25" t="n">
+        <v>530.1319999999999</v>
+      </c>
+      <c r="F25" t="n">
+        <v>75.474</v>
+      </c>
+      <c r="G25" t="n">
+        <v>53.354</v>
+      </c>
+      <c r="H25" t="n">
+        <v>79.49299999999999</v>
+      </c>
+      <c r="I25" t="n">
+        <v>4.46</v>
+      </c>
+      <c r="J25" t="n">
+        <v>3.666</v>
+      </c>
+      <c r="K25" t="n">
+        <v>300.299</v>
+      </c>
+      <c r="L25" t="n">
+        <v>259.246</v>
+      </c>
+      <c r="M25" t="n">
+        <v>0</v>
+      </c>
+      <c r="N25" t="n">
+        <v>3.923</v>
+      </c>
+      <c r="O25" t="n">
+        <v>0</v>
+      </c>
+      <c r="P25" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q25" t="n">
+        <v>0.14</v>
+      </c>
+      <c r="R25" t="n">
+        <v>0</v>
+      </c>
+      <c r="S25" t="n">
+        <v>0.645</v>
+      </c>
+      <c r="T25" t="n">
+        <v>6.022</v>
+      </c>
+      <c r="U25" t="n">
+        <v>0.754</v>
+      </c>
+      <c r="V25" t="n">
+        <v>79.49299999999999</v>
+      </c>
+      <c r="W25" t="n">
+        <v>0.754</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>20</v>
+      </c>
+      <c r="B26" t="n">
+        <v>348.093</v>
+      </c>
+      <c r="C26" t="n">
+        <v>237.63</v>
+      </c>
+      <c r="D26" t="n">
+        <v>45.878</v>
+      </c>
+      <c r="E26" t="n">
+        <v>530.1319999999999</v>
+      </c>
+      <c r="F26" t="n">
+        <v>75.474</v>
+      </c>
+      <c r="G26" t="n">
+        <v>58.164</v>
+      </c>
+      <c r="H26" t="n">
+        <v>85.092</v>
+      </c>
+      <c r="I26" t="n">
+        <v>4.46</v>
+      </c>
+      <c r="J26" t="n">
+        <v>3.666</v>
+      </c>
+      <c r="K26" t="n">
+        <v>300.409</v>
+      </c>
+      <c r="L26" t="n">
+        <v>261.507</v>
+      </c>
+      <c r="M26" t="n">
+        <v>0</v>
+      </c>
+      <c r="N26" t="n">
+        <v>3.923</v>
+      </c>
+      <c r="O26" t="n">
+        <v>0</v>
+      </c>
+      <c r="P26" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q26" t="n">
+        <v>0.14</v>
+      </c>
+      <c r="R26" t="n">
+        <v>0</v>
+      </c>
+      <c r="S26" t="n">
+        <v>0.645</v>
+      </c>
+      <c r="T26" t="n">
+        <v>6.022</v>
+      </c>
+      <c r="U26" t="n">
+        <v>0.754</v>
+      </c>
+      <c r="V26" t="n">
+        <v>85.092</v>
+      </c>
+      <c r="W26" t="n">
+        <v>0.754</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>21</v>
+      </c>
+      <c r="B27" t="n">
+        <v>358.168</v>
+      </c>
+      <c r="C27" t="n">
+        <v>374.324</v>
+      </c>
+      <c r="D27" t="n">
+        <v>45.878</v>
+      </c>
+      <c r="E27" t="n">
+        <v>568.165</v>
+      </c>
+      <c r="F27" t="n">
+        <v>82.17100000000001</v>
+      </c>
+      <c r="G27" t="n">
+        <v>58.164</v>
+      </c>
+      <c r="H27" t="n">
+        <v>87.72799999999999</v>
+      </c>
+      <c r="I27" t="n">
+        <v>4.46</v>
+      </c>
+      <c r="J27" t="n">
+        <v>3.666</v>
+      </c>
+      <c r="K27" t="n">
+        <v>303.729</v>
+      </c>
+      <c r="L27" t="n">
+        <v>262.823</v>
+      </c>
+      <c r="M27" t="n">
+        <v>0</v>
+      </c>
+      <c r="N27" t="n">
+        <v>3.923</v>
+      </c>
+      <c r="O27" t="n">
+        <v>0</v>
+      </c>
+      <c r="P27" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q27" t="n">
+        <v>0.439</v>
+      </c>
+      <c r="R27" t="n">
+        <v>0</v>
+      </c>
+      <c r="S27" t="n">
+        <v>0.645</v>
+      </c>
+      <c r="T27" t="n">
+        <v>6.949</v>
+      </c>
+      <c r="U27" t="n">
+        <v>0.754</v>
+      </c>
+      <c r="V27" t="n">
+        <v>87.72799999999999</v>
+      </c>
+      <c r="W27" t="n">
+        <v>0.754</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="1" t="inlineStr">
+        <is>
+          <t>STATISTICS TO RUN IN PRISM</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  The curves are descriptive. Test the ENDPOINT (day 21 total) only:</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Analyze → Column analyses → t test (and nonparametric tests)</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">         → 'Mann-Whitney test' (unpaired, two-tailed), EGFP vs SV2A.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  EXPECTED: median EGFP 87.7 min, SV2A 0.8 min, p = 0.0032</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Do not run a 2-way ANOVA over days: cumulative values are not</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  independent across time, so the day factor is not interpretable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="3" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="3" t="inlineStr">
+        <is>
+          <t>PLOT MEDIAN, NOT MEAN +/- SEM. The SV2A group is bimodal — 4 animals</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="3" t="inlineStr">
+        <is>
+          <t>at exactly 0 for all 21 days and 2 non-responders as high as EGFP — so</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="3" t="inlineStr">
+        <is>
+          <t>the mean is dragged up and the error bars overlap (EGFP 225 +/- 78 vs</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="3" t="inlineStr">
+        <is>
+          <t>SV2A 45 +/- 29 min), which understates a difference the medians show</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="3" t="inlineStr">
+        <is>
+          <t>clearly (87.7 vs 0.8 min).</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="3" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="3" t="inlineStr">
+        <is>
+          <t>ZEROS ARE REAL. A flat line along the axis means that animal never had</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="3" t="inlineStr">
+        <is>
+          <t>a seizure; it is not a plotting floor. Use a LINEAR y-axis here — do not</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="3" t="inlineStr">
+        <is>
+          <t>log-transform, or the flat-at-zero animals cannot be drawn.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="3" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="3" t="inlineStr">
+        <is>
+          <t>NON-RESPONDERS: SV2A animals with the two highest totals are the two</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="3" t="inlineStr">
+        <is>
+          <t>climbing SV2A lines; naming them in the legend is worth doing, since the</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="3" t="inlineStr">
+        <is>
+          <t>responder/non-responder split is more informative than the group median.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Cumulative-burden sheet: split convulsive-only from all seizures
The y-axis question was ambiguous — the sheet summed both seizure types
without saying so. Now writes two labelled blocks.

Convulsive-only is recommended: its 5/13 SV2A animals that never seize are the
same animals censored in the survival panel, so the two new panels
cross-reference. All-seizures gives 4/13 at zero, which a reader would then
have to reconcile against the survival curve. Convulsive-only also tests
slightly stronger (p = 0.0018 vs 0.0032).

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Figure3_replacement_panels.xlsx
+++ b/Figure3_replacement_panels.xlsx
@@ -1263,7 +1263,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W49"/>
+  <dimension ref="A1:W78"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -1301,211 +1301,147 @@
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>PRISM TABLE TYPE:  XY, with X = day and one Y column per animal (Y = single values, no replicates)</t>
+          <t>PRISM TABLE TYPE:  XY, X = day, one Y column per animal (Y = single values, no replicates)</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Plot every animal as a thin grey line; overlay the two group MEDIAN columns as bold lines. Do not use mean +/- SEM — see note.</t>
+          <t>Two blocks below: CONVULSIVE ONLY and ALL SEIZURES. Use one. Plot each animal as a thin grey line, group medians bold.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr">
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>BLOCK 1 — CONVULSIVE seizures only (recommended: matches the survival panel)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
         <is>
           <t>X  (day)</t>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="B7" s="2" t="inlineStr">
         <is>
           <t>EGFP 25</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr">
+      <c r="C7" s="2" t="inlineStr">
         <is>
           <t>EGFP 31</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr">
+      <c r="D7" s="2" t="inlineStr">
         <is>
           <t>EGFP 33</t>
         </is>
       </c>
-      <c r="E6" s="2" t="inlineStr">
+      <c r="E7" s="2" t="inlineStr">
         <is>
           <t>EGFP 355675</t>
         </is>
       </c>
-      <c r="F6" s="2" t="inlineStr">
+      <c r="F7" s="2" t="inlineStr">
         <is>
           <t>EGFP 355679</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr">
+      <c r="G7" s="2" t="inlineStr">
         <is>
           <t>EGFP 372833</t>
         </is>
       </c>
-      <c r="H6" s="2" t="inlineStr">
+      <c r="H7" s="2" t="inlineStr">
         <is>
           <t>EGFP 372838</t>
         </is>
       </c>
-      <c r="I6" s="2" t="inlineStr">
+      <c r="I7" s="2" t="inlineStr">
         <is>
           <t>SV2A 24</t>
         </is>
       </c>
-      <c r="J6" s="2" t="inlineStr">
+      <c r="J7" s="2" t="inlineStr">
         <is>
           <t>SV2A 26</t>
         </is>
       </c>
-      <c r="K6" s="2" t="inlineStr">
+      <c r="K7" s="2" t="inlineStr">
         <is>
           <t>SV2A 29</t>
         </is>
       </c>
-      <c r="L6" s="2" t="inlineStr">
+      <c r="L7" s="2" t="inlineStr">
         <is>
           <t>SV2A 32</t>
         </is>
       </c>
-      <c r="M6" s="2" t="inlineStr">
+      <c r="M7" s="2" t="inlineStr">
         <is>
           <t>SV2A 355668</t>
         </is>
       </c>
-      <c r="N6" s="2" t="inlineStr">
+      <c r="N7" s="2" t="inlineStr">
         <is>
           <t>SV2A 355669</t>
         </is>
       </c>
-      <c r="O6" s="2" t="inlineStr">
+      <c r="O7" s="2" t="inlineStr">
         <is>
           <t>SV2A 355670</t>
         </is>
       </c>
-      <c r="P6" s="2" t="inlineStr">
+      <c r="P7" s="2" t="inlineStr">
         <is>
           <t>SV2A 355673</t>
         </is>
       </c>
-      <c r="Q6" s="2" t="inlineStr">
+      <c r="Q7" s="2" t="inlineStr">
         <is>
           <t>SV2A 355677</t>
         </is>
       </c>
-      <c r="R6" s="2" t="inlineStr">
+      <c r="R7" s="2" t="inlineStr">
         <is>
           <t>SV2A 372828</t>
         </is>
       </c>
-      <c r="S6" s="2" t="inlineStr">
+      <c r="S7" s="2" t="inlineStr">
         <is>
           <t>SV2A 372829</t>
         </is>
       </c>
-      <c r="T6" s="2" t="inlineStr">
+      <c r="T7" s="2" t="inlineStr">
         <is>
           <t>SV2A 372830</t>
         </is>
       </c>
-      <c r="U6" s="2" t="inlineStr">
+      <c r="U7" s="2" t="inlineStr">
         <is>
           <t>SV2A 372832</t>
         </is>
       </c>
-      <c r="V6" s="2" t="inlineStr">
+      <c r="V7" s="2" t="inlineStr">
         <is>
           <t>EGFP median</t>
         </is>
       </c>
-      <c r="W6" s="2" t="inlineStr">
+      <c r="W7" s="2" t="inlineStr">
         <is>
           <t>SV2A median</t>
         </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="n">
-        <v>1</v>
-      </c>
-      <c r="B7" t="n">
-        <v>3.777</v>
-      </c>
-      <c r="C7" t="n">
-        <v>0</v>
-      </c>
-      <c r="D7" t="n">
-        <v>0</v>
-      </c>
-      <c r="E7" t="n">
-        <v>8.137</v>
-      </c>
-      <c r="F7" t="n">
-        <v>4.501</v>
-      </c>
-      <c r="G7" t="n">
-        <v>0</v>
-      </c>
-      <c r="H7" t="n">
-        <v>0</v>
-      </c>
-      <c r="I7" t="n">
-        <v>0</v>
-      </c>
-      <c r="J7" t="n">
-        <v>1.174</v>
-      </c>
-      <c r="K7" t="n">
-        <v>17.018</v>
-      </c>
-      <c r="L7" t="n">
-        <v>2.981</v>
-      </c>
-      <c r="M7" t="n">
-        <v>0</v>
-      </c>
-      <c r="N7" t="n">
-        <v>0</v>
-      </c>
-      <c r="O7" t="n">
-        <v>0</v>
-      </c>
-      <c r="P7" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q7" t="n">
-        <v>0</v>
-      </c>
-      <c r="R7" t="n">
-        <v>0</v>
-      </c>
-      <c r="S7" t="n">
-        <v>0</v>
-      </c>
-      <c r="T7" t="n">
-        <v>0</v>
-      </c>
-      <c r="U7" t="n">
-        <v>0</v>
-      </c>
-      <c r="V7" t="n">
-        <v>0</v>
-      </c>
-      <c r="W7" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B8" t="n">
-        <v>5.25</v>
+        <v>3.777</v>
       </c>
       <c r="C8" t="n">
         <v>0</v>
@@ -1514,28 +1450,28 @@
         <v>0</v>
       </c>
       <c r="E8" t="n">
-        <v>23.419</v>
+        <v>0.304</v>
       </c>
       <c r="F8" t="n">
-        <v>7.226</v>
+        <v>3.873</v>
       </c>
       <c r="G8" t="n">
-        <v>1.865</v>
+        <v>0</v>
       </c>
       <c r="H8" t="n">
-        <v>8.156000000000001</v>
+        <v>0</v>
       </c>
       <c r="I8" t="n">
         <v>0</v>
       </c>
       <c r="J8" t="n">
-        <v>1.278</v>
+        <v>1.174</v>
       </c>
       <c r="K8" t="n">
-        <v>22.114</v>
+        <v>1.874</v>
       </c>
       <c r="L8" t="n">
-        <v>5.109</v>
+        <v>2.538</v>
       </c>
       <c r="M8" t="n">
         <v>0</v>
@@ -1565,7 +1501,7 @@
         <v>0</v>
       </c>
       <c r="V8" t="n">
-        <v>5.25</v>
+        <v>0</v>
       </c>
       <c r="W8" t="n">
         <v>0</v>
@@ -1573,10 +1509,10 @@
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B9" t="n">
-        <v>6.235</v>
+        <v>5.25</v>
       </c>
       <c r="C9" t="n">
         <v>0</v>
@@ -1585,34 +1521,34 @@
         <v>0</v>
       </c>
       <c r="E9" t="n">
-        <v>41.704</v>
+        <v>4.511</v>
       </c>
       <c r="F9" t="n">
-        <v>11.329</v>
+        <v>4.615</v>
       </c>
       <c r="G9" t="n">
-        <v>3.768</v>
+        <v>1.865</v>
       </c>
       <c r="H9" t="n">
-        <v>10.328</v>
+        <v>6.569</v>
       </c>
       <c r="I9" t="n">
         <v>0</v>
       </c>
       <c r="J9" t="n">
-        <v>1.278</v>
+        <v>1.174</v>
       </c>
       <c r="K9" t="n">
-        <v>30.063</v>
+        <v>3.488</v>
       </c>
       <c r="L9" t="n">
-        <v>9.436999999999999</v>
+        <v>4.666</v>
       </c>
       <c r="M9" t="n">
         <v>0</v>
       </c>
       <c r="N9" t="n">
-        <v>0.261</v>
+        <v>0</v>
       </c>
       <c r="O9" t="n">
         <v>0</v>
@@ -1627,16 +1563,16 @@
         <v>0</v>
       </c>
       <c r="S9" t="n">
-        <v>0.436</v>
+        <v>0</v>
       </c>
       <c r="T9" t="n">
-        <v>0.626</v>
+        <v>0</v>
       </c>
       <c r="U9" t="n">
         <v>0</v>
       </c>
       <c r="V9" t="n">
-        <v>6.235</v>
+        <v>4.511</v>
       </c>
       <c r="W9" t="n">
         <v>0</v>
@@ -1644,46 +1580,46 @@
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B10" t="n">
-        <v>9.663</v>
+        <v>5.837</v>
       </c>
       <c r="C10" t="n">
-        <v>2.561</v>
+        <v>0</v>
       </c>
       <c r="D10" t="n">
         <v>0</v>
       </c>
       <c r="E10" t="n">
-        <v>61.922</v>
+        <v>17.72</v>
       </c>
       <c r="F10" t="n">
-        <v>18.563</v>
+        <v>5.824</v>
       </c>
       <c r="G10" t="n">
-        <v>6.413</v>
+        <v>3.768</v>
       </c>
       <c r="H10" t="n">
-        <v>13.633</v>
+        <v>8.25</v>
       </c>
       <c r="I10" t="n">
-        <v>1.317</v>
+        <v>0</v>
       </c>
       <c r="J10" t="n">
-        <v>1.598</v>
+        <v>1.174</v>
       </c>
       <c r="K10" t="n">
-        <v>37.563</v>
+        <v>6.659</v>
       </c>
       <c r="L10" t="n">
-        <v>18.395</v>
+        <v>8.994</v>
       </c>
       <c r="M10" t="n">
         <v>0</v>
       </c>
       <c r="N10" t="n">
-        <v>0.261</v>
+        <v>0</v>
       </c>
       <c r="O10" t="n">
         <v>0</v>
@@ -1698,7 +1634,7 @@
         <v>0</v>
       </c>
       <c r="S10" t="n">
-        <v>0.645</v>
+        <v>0</v>
       </c>
       <c r="T10" t="n">
         <v>0.626</v>
@@ -1707,54 +1643,54 @@
         <v>0</v>
       </c>
       <c r="V10" t="n">
-        <v>9.663</v>
+        <v>5.824</v>
       </c>
       <c r="W10" t="n">
-        <v>0.261</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B11" t="n">
-        <v>13.277</v>
+        <v>9.145</v>
       </c>
       <c r="C11" t="n">
-        <v>3.493</v>
+        <v>0</v>
       </c>
       <c r="D11" t="n">
         <v>0</v>
       </c>
       <c r="E11" t="n">
-        <v>107.61</v>
+        <v>30.024</v>
       </c>
       <c r="F11" t="n">
-        <v>30.952</v>
+        <v>10.022</v>
       </c>
       <c r="G11" t="n">
-        <v>10.624</v>
+        <v>6.413</v>
       </c>
       <c r="H11" t="n">
-        <v>31.862</v>
+        <v>9.336</v>
       </c>
       <c r="I11" t="n">
         <v>1.317</v>
       </c>
       <c r="J11" t="n">
-        <v>1.598</v>
+        <v>1.174</v>
       </c>
       <c r="K11" t="n">
-        <v>40.302</v>
+        <v>13.729</v>
       </c>
       <c r="L11" t="n">
-        <v>25.484</v>
+        <v>17.952</v>
       </c>
       <c r="M11" t="n">
         <v>0</v>
       </c>
       <c r="N11" t="n">
-        <v>0.779</v>
+        <v>0</v>
       </c>
       <c r="O11" t="n">
         <v>0</v>
@@ -1769,7 +1705,7 @@
         <v>0</v>
       </c>
       <c r="S11" t="n">
-        <v>0.645</v>
+        <v>0</v>
       </c>
       <c r="T11" t="n">
         <v>0.626</v>
@@ -1778,54 +1714,54 @@
         <v>0</v>
       </c>
       <c r="V11" t="n">
-        <v>13.277</v>
+        <v>9.145</v>
       </c>
       <c r="W11" t="n">
-        <v>0.626</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B12" t="n">
-        <v>18.357</v>
+        <v>12.652</v>
       </c>
       <c r="C12" t="n">
-        <v>6.629</v>
+        <v>0</v>
       </c>
       <c r="D12" t="n">
         <v>0</v>
       </c>
       <c r="E12" t="n">
-        <v>107.61</v>
+        <v>48.474</v>
       </c>
       <c r="F12" t="n">
-        <v>30.952</v>
+        <v>17.707</v>
       </c>
       <c r="G12" t="n">
         <v>10.624</v>
       </c>
       <c r="H12" t="n">
-        <v>31.862</v>
+        <v>26.851</v>
       </c>
       <c r="I12" t="n">
         <v>1.317</v>
       </c>
       <c r="J12" t="n">
-        <v>1.598</v>
+        <v>1.174</v>
       </c>
       <c r="K12" t="n">
-        <v>45.075</v>
+        <v>16.172</v>
       </c>
       <c r="L12" t="n">
-        <v>45.433</v>
+        <v>25.041</v>
       </c>
       <c r="M12" t="n">
         <v>0</v>
       </c>
       <c r="N12" t="n">
-        <v>0.779</v>
+        <v>0.518</v>
       </c>
       <c r="O12" t="n">
         <v>0</v>
@@ -1840,7 +1776,7 @@
         <v>0</v>
       </c>
       <c r="S12" t="n">
-        <v>0.645</v>
+        <v>0</v>
       </c>
       <c r="T12" t="n">
         <v>0.626</v>
@@ -1849,54 +1785,54 @@
         <v>0</v>
       </c>
       <c r="V12" t="n">
-        <v>18.357</v>
+        <v>12.652</v>
       </c>
       <c r="W12" t="n">
-        <v>0.626</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B13" t="n">
-        <v>22.407</v>
+        <v>17.337</v>
       </c>
       <c r="C13" t="n">
-        <v>9.331</v>
+        <v>0</v>
       </c>
       <c r="D13" t="n">
         <v>0</v>
       </c>
       <c r="E13" t="n">
-        <v>126.484</v>
+        <v>48.474</v>
       </c>
       <c r="F13" t="n">
-        <v>33.083</v>
+        <v>17.707</v>
       </c>
       <c r="G13" t="n">
-        <v>14.536</v>
+        <v>10.624</v>
       </c>
       <c r="H13" t="n">
-        <v>36.628</v>
+        <v>26.851</v>
       </c>
       <c r="I13" t="n">
         <v>1.317</v>
       </c>
       <c r="J13" t="n">
-        <v>1.598</v>
+        <v>1.174</v>
       </c>
       <c r="K13" t="n">
-        <v>67.09999999999999</v>
+        <v>16.172</v>
       </c>
       <c r="L13" t="n">
-        <v>63.464</v>
+        <v>44.99</v>
       </c>
       <c r="M13" t="n">
         <v>0</v>
       </c>
       <c r="N13" t="n">
-        <v>0.779</v>
+        <v>0.518</v>
       </c>
       <c r="O13" t="n">
         <v>0</v>
@@ -1911,63 +1847,63 @@
         <v>0</v>
       </c>
       <c r="S13" t="n">
-        <v>0.645</v>
+        <v>0</v>
       </c>
       <c r="T13" t="n">
-        <v>1.276</v>
+        <v>0.626</v>
       </c>
       <c r="U13" t="n">
         <v>0</v>
       </c>
       <c r="V13" t="n">
-        <v>22.407</v>
+        <v>17.337</v>
       </c>
       <c r="W13" t="n">
-        <v>0.645</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B14" t="n">
-        <v>28.332</v>
+        <v>20.797</v>
       </c>
       <c r="C14" t="n">
-        <v>13.248</v>
+        <v>0</v>
       </c>
       <c r="D14" t="n">
         <v>0</v>
       </c>
       <c r="E14" t="n">
-        <v>158.689</v>
+        <v>52.596</v>
       </c>
       <c r="F14" t="n">
-        <v>40.131</v>
+        <v>18.552</v>
       </c>
       <c r="G14" t="n">
-        <v>18.88</v>
+        <v>14.536</v>
       </c>
       <c r="H14" t="n">
-        <v>36.628</v>
+        <v>31.616</v>
       </c>
       <c r="I14" t="n">
         <v>1.317</v>
       </c>
       <c r="J14" t="n">
-        <v>1.598</v>
+        <v>1.174</v>
       </c>
       <c r="K14" t="n">
-        <v>111.623</v>
+        <v>16.172</v>
       </c>
       <c r="L14" t="n">
-        <v>81.935</v>
+        <v>63.021</v>
       </c>
       <c r="M14" t="n">
         <v>0</v>
       </c>
       <c r="N14" t="n">
-        <v>0.889</v>
+        <v>0.518</v>
       </c>
       <c r="O14" t="n">
         <v>0</v>
@@ -1982,63 +1918,63 @@
         <v>0</v>
       </c>
       <c r="S14" t="n">
-        <v>0.645</v>
+        <v>0</v>
       </c>
       <c r="T14" t="n">
-        <v>2.044</v>
+        <v>1.276</v>
       </c>
       <c r="U14" t="n">
         <v>0</v>
       </c>
       <c r="V14" t="n">
-        <v>28.332</v>
+        <v>18.552</v>
       </c>
       <c r="W14" t="n">
-        <v>0.645</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B15" t="n">
-        <v>33.647</v>
+        <v>25.768</v>
       </c>
       <c r="C15" t="n">
-        <v>18.568</v>
+        <v>1.263</v>
       </c>
       <c r="D15" t="n">
-        <v>0.256</v>
+        <v>0</v>
       </c>
       <c r="E15" t="n">
-        <v>194.037</v>
+        <v>63.902</v>
       </c>
       <c r="F15" t="n">
-        <v>44.558</v>
+        <v>22.387</v>
       </c>
       <c r="G15" t="n">
-        <v>20.52</v>
+        <v>18.88</v>
       </c>
       <c r="H15" t="n">
-        <v>37.625</v>
+        <v>31.616</v>
       </c>
       <c r="I15" t="n">
         <v>1.317</v>
       </c>
       <c r="J15" t="n">
-        <v>1.598</v>
+        <v>1.174</v>
       </c>
       <c r="K15" t="n">
-        <v>144.082</v>
+        <v>17.157</v>
       </c>
       <c r="L15" t="n">
-        <v>103.187</v>
+        <v>81.492</v>
       </c>
       <c r="M15" t="n">
         <v>0</v>
       </c>
       <c r="N15" t="n">
-        <v>0.889</v>
+        <v>0.628</v>
       </c>
       <c r="O15" t="n">
         <v>0</v>
@@ -2053,7 +1989,7 @@
         <v>0</v>
       </c>
       <c r="S15" t="n">
-        <v>0.645</v>
+        <v>0</v>
       </c>
       <c r="T15" t="n">
         <v>2.044</v>
@@ -2062,54 +1998,54 @@
         <v>0</v>
       </c>
       <c r="V15" t="n">
-        <v>33.647</v>
+        <v>22.387</v>
       </c>
       <c r="W15" t="n">
-        <v>0.645</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B16" t="n">
-        <v>42.312</v>
+        <v>30.76</v>
       </c>
       <c r="C16" t="n">
-        <v>24.996</v>
+        <v>3.211</v>
       </c>
       <c r="D16" t="n">
-        <v>0.756</v>
+        <v>0.108</v>
       </c>
       <c r="E16" t="n">
-        <v>251.443</v>
+        <v>72.517</v>
       </c>
       <c r="F16" t="n">
-        <v>46.512</v>
+        <v>25.188</v>
       </c>
       <c r="G16" t="n">
-        <v>22.846</v>
+        <v>20.52</v>
       </c>
       <c r="H16" t="n">
-        <v>46.251</v>
+        <v>31.616</v>
       </c>
       <c r="I16" t="n">
-        <v>2.835</v>
+        <v>1.317</v>
       </c>
       <c r="J16" t="n">
-        <v>1.598</v>
+        <v>1.174</v>
       </c>
       <c r="K16" t="n">
-        <v>160.912</v>
+        <v>19.906</v>
       </c>
       <c r="L16" t="n">
-        <v>119.698</v>
+        <v>102.744</v>
       </c>
       <c r="M16" t="n">
         <v>0</v>
       </c>
       <c r="N16" t="n">
-        <v>1.704</v>
+        <v>0.628</v>
       </c>
       <c r="O16" t="n">
         <v>0</v>
@@ -2124,63 +2060,63 @@
         <v>0</v>
       </c>
       <c r="S16" t="n">
-        <v>0.645</v>
+        <v>0</v>
       </c>
       <c r="T16" t="n">
-        <v>2.488</v>
+        <v>2.044</v>
       </c>
       <c r="U16" t="n">
         <v>0</v>
       </c>
       <c r="V16" t="n">
-        <v>42.312</v>
+        <v>25.188</v>
       </c>
       <c r="W16" t="n">
-        <v>0.645</v>
+        <v>0</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B17" t="n">
-        <v>60.44</v>
+        <v>38.962</v>
       </c>
       <c r="C17" t="n">
-        <v>35.622</v>
+        <v>5.066</v>
       </c>
       <c r="D17" t="n">
-        <v>4.661</v>
+        <v>0.609</v>
       </c>
       <c r="E17" t="n">
-        <v>251.443</v>
+        <v>79.669</v>
       </c>
       <c r="F17" t="n">
-        <v>46.512</v>
+        <v>25.878</v>
       </c>
       <c r="G17" t="n">
-        <v>27.772</v>
+        <v>22.846</v>
       </c>
       <c r="H17" t="n">
-        <v>51.071</v>
+        <v>39.334</v>
       </c>
       <c r="I17" t="n">
-        <v>3.798</v>
+        <v>2.835</v>
       </c>
       <c r="J17" t="n">
-        <v>3.046</v>
+        <v>1.174</v>
       </c>
       <c r="K17" t="n">
-        <v>189.689</v>
+        <v>19.906</v>
       </c>
       <c r="L17" t="n">
-        <v>151.666</v>
+        <v>118.428</v>
       </c>
       <c r="M17" t="n">
         <v>0</v>
       </c>
       <c r="N17" t="n">
-        <v>1.704</v>
+        <v>1.166</v>
       </c>
       <c r="O17" t="n">
         <v>0</v>
@@ -2195,7 +2131,7 @@
         <v>0</v>
       </c>
       <c r="S17" t="n">
-        <v>0.645</v>
+        <v>0</v>
       </c>
       <c r="T17" t="n">
         <v>2.488</v>
@@ -2204,54 +2140,54 @@
         <v>0</v>
       </c>
       <c r="V17" t="n">
-        <v>46.512</v>
+        <v>25.878</v>
       </c>
       <c r="W17" t="n">
-        <v>0.645</v>
+        <v>0</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B18" t="n">
-        <v>67.619</v>
+        <v>55.988</v>
       </c>
       <c r="C18" t="n">
-        <v>40.11</v>
+        <v>10.124</v>
       </c>
       <c r="D18" t="n">
-        <v>9.643000000000001</v>
+        <v>4.514</v>
       </c>
       <c r="E18" t="n">
-        <v>280.865</v>
+        <v>79.669</v>
       </c>
       <c r="F18" t="n">
-        <v>52.65</v>
+        <v>25.878</v>
       </c>
       <c r="G18" t="n">
-        <v>37.209</v>
+        <v>27.772</v>
       </c>
       <c r="H18" t="n">
-        <v>58.696</v>
+        <v>44.154</v>
       </c>
       <c r="I18" t="n">
-        <v>4.46</v>
+        <v>3.798</v>
       </c>
       <c r="J18" t="n">
-        <v>3.666</v>
+        <v>2.622</v>
       </c>
       <c r="K18" t="n">
-        <v>212.859</v>
+        <v>22.738</v>
       </c>
       <c r="L18" t="n">
-        <v>168.506</v>
+        <v>147.713</v>
       </c>
       <c r="M18" t="n">
         <v>0</v>
       </c>
       <c r="N18" t="n">
-        <v>1.704</v>
+        <v>1.166</v>
       </c>
       <c r="O18" t="n">
         <v>0</v>
@@ -2266,63 +2202,63 @@
         <v>0</v>
       </c>
       <c r="S18" t="n">
-        <v>0.645</v>
+        <v>0</v>
       </c>
       <c r="T18" t="n">
-        <v>3.557</v>
+        <v>2.488</v>
       </c>
       <c r="U18" t="n">
         <v>0</v>
       </c>
       <c r="V18" t="n">
-        <v>52.65</v>
+        <v>27.772</v>
       </c>
       <c r="W18" t="n">
-        <v>0.645</v>
+        <v>0</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B19" t="n">
-        <v>80.44799999999999</v>
+        <v>61.921</v>
       </c>
       <c r="C19" t="n">
-        <v>46.453</v>
+        <v>11.799</v>
       </c>
       <c r="D19" t="n">
-        <v>16.988</v>
+        <v>9.494999999999999</v>
       </c>
       <c r="E19" t="n">
-        <v>323.538</v>
+        <v>80.127</v>
       </c>
       <c r="F19" t="n">
-        <v>57.78</v>
+        <v>29.302</v>
       </c>
       <c r="G19" t="n">
         <v>37.209</v>
       </c>
       <c r="H19" t="n">
-        <v>58.696</v>
+        <v>51.173</v>
       </c>
       <c r="I19" t="n">
         <v>4.46</v>
       </c>
       <c r="J19" t="n">
-        <v>3.666</v>
+        <v>3.242</v>
       </c>
       <c r="K19" t="n">
-        <v>230.531</v>
+        <v>25.782</v>
       </c>
       <c r="L19" t="n">
-        <v>187.336</v>
+        <v>163.624</v>
       </c>
       <c r="M19" t="n">
         <v>0</v>
       </c>
       <c r="N19" t="n">
-        <v>2.314</v>
+        <v>1.166</v>
       </c>
       <c r="O19" t="n">
         <v>0</v>
@@ -2337,7 +2273,7 @@
         <v>0</v>
       </c>
       <c r="S19" t="n">
-        <v>0.645</v>
+        <v>0</v>
       </c>
       <c r="T19" t="n">
         <v>3.557</v>
@@ -2346,54 +2282,54 @@
         <v>0</v>
       </c>
       <c r="V19" t="n">
-        <v>57.78</v>
+        <v>37.209</v>
       </c>
       <c r="W19" t="n">
-        <v>0.645</v>
+        <v>0</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B20" t="n">
-        <v>90.556</v>
+        <v>74.199</v>
       </c>
       <c r="C20" t="n">
-        <v>52.48</v>
+        <v>15.141</v>
       </c>
       <c r="D20" t="n">
-        <v>22.657</v>
+        <v>16.84</v>
       </c>
       <c r="E20" t="n">
-        <v>323.538</v>
+        <v>82.709</v>
       </c>
       <c r="F20" t="n">
-        <v>57.78</v>
+        <v>31.118</v>
       </c>
       <c r="G20" t="n">
-        <v>40.414</v>
+        <v>37.209</v>
       </c>
       <c r="H20" t="n">
-        <v>61.623</v>
+        <v>51.173</v>
       </c>
       <c r="I20" t="n">
         <v>4.46</v>
       </c>
       <c r="J20" t="n">
-        <v>3.666</v>
+        <v>3.242</v>
       </c>
       <c r="K20" t="n">
-        <v>269.418</v>
+        <v>25.879</v>
       </c>
       <c r="L20" t="n">
-        <v>201.509</v>
+        <v>181.079</v>
       </c>
       <c r="M20" t="n">
         <v>0</v>
       </c>
       <c r="N20" t="n">
-        <v>2.314</v>
+        <v>1.255</v>
       </c>
       <c r="O20" t="n">
         <v>0</v>
@@ -2408,7 +2344,7 @@
         <v>0</v>
       </c>
       <c r="S20" t="n">
-        <v>0.645</v>
+        <v>0</v>
       </c>
       <c r="T20" t="n">
         <v>3.557</v>
@@ -2417,54 +2353,54 @@
         <v>0</v>
       </c>
       <c r="V20" t="n">
-        <v>57.78</v>
+        <v>37.209</v>
       </c>
       <c r="W20" t="n">
-        <v>0.645</v>
+        <v>0</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B21" t="n">
-        <v>123.142</v>
+        <v>83.628</v>
       </c>
       <c r="C21" t="n">
-        <v>65.702</v>
+        <v>18.686</v>
       </c>
       <c r="D21" t="n">
-        <v>31.719</v>
+        <v>22.31</v>
       </c>
       <c r="E21" t="n">
-        <v>351.599</v>
+        <v>82.709</v>
       </c>
       <c r="F21" t="n">
-        <v>60.956</v>
+        <v>31.118</v>
       </c>
       <c r="G21" t="n">
-        <v>44.871</v>
+        <v>40.414</v>
       </c>
       <c r="H21" t="n">
-        <v>64.04600000000001</v>
+        <v>54.1</v>
       </c>
       <c r="I21" t="n">
         <v>4.46</v>
       </c>
       <c r="J21" t="n">
-        <v>3.666</v>
+        <v>3.242</v>
       </c>
       <c r="K21" t="n">
-        <v>274.214</v>
+        <v>27.472</v>
       </c>
       <c r="L21" t="n">
-        <v>226.165</v>
+        <v>195.014</v>
       </c>
       <c r="M21" t="n">
         <v>0</v>
       </c>
       <c r="N21" t="n">
-        <v>2.314</v>
+        <v>1.255</v>
       </c>
       <c r="O21" t="n">
         <v>0</v>
@@ -2479,7 +2415,7 @@
         <v>0</v>
       </c>
       <c r="S21" t="n">
-        <v>0.645</v>
+        <v>0</v>
       </c>
       <c r="T21" t="n">
         <v>3.557</v>
@@ -2488,54 +2424,54 @@
         <v>0</v>
       </c>
       <c r="V21" t="n">
-        <v>64.04600000000001</v>
+        <v>40.414</v>
       </c>
       <c r="W21" t="n">
-        <v>0.645</v>
+        <v>0</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B22" t="n">
-        <v>193.203</v>
+        <v>110.095</v>
       </c>
       <c r="C22" t="n">
-        <v>72.986</v>
+        <v>26.705</v>
       </c>
       <c r="D22" t="n">
-        <v>38.706</v>
+        <v>31.371</v>
       </c>
       <c r="E22" t="n">
-        <v>392.31</v>
+        <v>84.88200000000001</v>
       </c>
       <c r="F22" t="n">
-        <v>62.511</v>
+        <v>32.81</v>
       </c>
       <c r="G22" t="n">
-        <v>47.128</v>
+        <v>44.871</v>
       </c>
       <c r="H22" t="n">
-        <v>67.16800000000001</v>
+        <v>56.523</v>
       </c>
       <c r="I22" t="n">
         <v>4.46</v>
       </c>
       <c r="J22" t="n">
-        <v>3.666</v>
+        <v>3.242</v>
       </c>
       <c r="K22" t="n">
-        <v>281.802</v>
+        <v>28.814</v>
       </c>
       <c r="L22" t="n">
-        <v>232.404</v>
+        <v>219.294</v>
       </c>
       <c r="M22" t="n">
         <v>0</v>
       </c>
       <c r="N22" t="n">
-        <v>2.314</v>
+        <v>1.255</v>
       </c>
       <c r="O22" t="n">
         <v>0</v>
@@ -2550,63 +2486,63 @@
         <v>0</v>
       </c>
       <c r="S22" t="n">
-        <v>0.645</v>
+        <v>0</v>
       </c>
       <c r="T22" t="n">
-        <v>4.415</v>
+        <v>3.557</v>
       </c>
       <c r="U22" t="n">
-        <v>0.539</v>
+        <v>0</v>
       </c>
       <c r="V22" t="n">
-        <v>67.16800000000001</v>
+        <v>44.871</v>
       </c>
       <c r="W22" t="n">
-        <v>0.645</v>
+        <v>0</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B23" t="n">
-        <v>245.679</v>
+        <v>170.98</v>
       </c>
       <c r="C23" t="n">
-        <v>85.22499999999999</v>
+        <v>30.539</v>
       </c>
       <c r="D23" t="n">
-        <v>45.181</v>
+        <v>38.359</v>
       </c>
       <c r="E23" t="n">
-        <v>435.401</v>
+        <v>90.622</v>
       </c>
       <c r="F23" t="n">
-        <v>65.43600000000001</v>
+        <v>33.487</v>
       </c>
       <c r="G23" t="n">
-        <v>48.834</v>
+        <v>46.911</v>
       </c>
       <c r="H23" t="n">
-        <v>70.408</v>
+        <v>59.645</v>
       </c>
       <c r="I23" t="n">
         <v>4.46</v>
       </c>
       <c r="J23" t="n">
-        <v>3.666</v>
+        <v>3.242</v>
       </c>
       <c r="K23" t="n">
-        <v>299.691</v>
+        <v>28.814</v>
       </c>
       <c r="L23" t="n">
-        <v>252.786</v>
+        <v>225.049</v>
       </c>
       <c r="M23" t="n">
         <v>0</v>
       </c>
       <c r="N23" t="n">
-        <v>2.314</v>
+        <v>1.255</v>
       </c>
       <c r="O23" t="n">
         <v>0</v>
@@ -2621,63 +2557,63 @@
         <v>0</v>
       </c>
       <c r="S23" t="n">
-        <v>0.645</v>
+        <v>0</v>
       </c>
       <c r="T23" t="n">
-        <v>5.465</v>
+        <v>4.415</v>
       </c>
       <c r="U23" t="n">
         <v>0.539</v>
       </c>
       <c r="V23" t="n">
-        <v>70.408</v>
+        <v>46.911</v>
       </c>
       <c r="W23" t="n">
-        <v>0.645</v>
+        <v>0.539</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B24" t="n">
-        <v>334.378</v>
+        <v>188.983</v>
       </c>
       <c r="C24" t="n">
-        <v>168.448</v>
+        <v>41.361</v>
       </c>
       <c r="D24" t="n">
-        <v>45.878</v>
+        <v>44.833</v>
       </c>
       <c r="E24" t="n">
-        <v>481.811</v>
+        <v>96.655</v>
       </c>
       <c r="F24" t="n">
-        <v>69.66800000000001</v>
+        <v>35.299</v>
       </c>
       <c r="G24" t="n">
-        <v>50.579</v>
+        <v>48.618</v>
       </c>
       <c r="H24" t="n">
-        <v>74.67</v>
+        <v>62.885</v>
       </c>
       <c r="I24" t="n">
         <v>4.46</v>
       </c>
       <c r="J24" t="n">
-        <v>3.666</v>
+        <v>3.242</v>
       </c>
       <c r="K24" t="n">
-        <v>300.299</v>
+        <v>32.231</v>
       </c>
       <c r="L24" t="n">
-        <v>259.246</v>
+        <v>244.938</v>
       </c>
       <c r="M24" t="n">
         <v>0</v>
       </c>
       <c r="N24" t="n">
-        <v>3.226</v>
+        <v>1.255</v>
       </c>
       <c r="O24" t="n">
         <v>0</v>
@@ -2692,7 +2628,7 @@
         <v>0</v>
       </c>
       <c r="S24" t="n">
-        <v>0.645</v>
+        <v>0</v>
       </c>
       <c r="T24" t="n">
         <v>5.465</v>
@@ -2701,54 +2637,54 @@
         <v>0.539</v>
       </c>
       <c r="V24" t="n">
-        <v>74.67</v>
+        <v>48.618</v>
       </c>
       <c r="W24" t="n">
-        <v>0.645</v>
+        <v>0.539</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B25" t="n">
-        <v>334.378</v>
+        <v>231.415</v>
       </c>
       <c r="C25" t="n">
-        <v>168.448</v>
+        <v>118.715</v>
       </c>
       <c r="D25" t="n">
-        <v>45.878</v>
+        <v>45.53</v>
       </c>
       <c r="E25" t="n">
-        <v>530.1319999999999</v>
+        <v>109.157</v>
       </c>
       <c r="F25" t="n">
-        <v>75.474</v>
+        <v>39.407</v>
       </c>
       <c r="G25" t="n">
-        <v>53.354</v>
+        <v>50.362</v>
       </c>
       <c r="H25" t="n">
-        <v>79.49299999999999</v>
+        <v>67.14700000000001</v>
       </c>
       <c r="I25" t="n">
         <v>4.46</v>
       </c>
       <c r="J25" t="n">
-        <v>3.666</v>
+        <v>3.242</v>
       </c>
       <c r="K25" t="n">
-        <v>300.299</v>
+        <v>32.838</v>
       </c>
       <c r="L25" t="n">
-        <v>259.246</v>
+        <v>250.054</v>
       </c>
       <c r="M25" t="n">
         <v>0</v>
       </c>
       <c r="N25" t="n">
-        <v>3.923</v>
+        <v>2.167</v>
       </c>
       <c r="O25" t="n">
         <v>0</v>
@@ -2757,69 +2693,69 @@
         <v>0</v>
       </c>
       <c r="Q25" t="n">
-        <v>0.14</v>
+        <v>0</v>
       </c>
       <c r="R25" t="n">
         <v>0</v>
       </c>
       <c r="S25" t="n">
-        <v>0.645</v>
+        <v>0</v>
       </c>
       <c r="T25" t="n">
-        <v>6.022</v>
+        <v>5.465</v>
       </c>
       <c r="U25" t="n">
-        <v>0.754</v>
+        <v>0.539</v>
       </c>
       <c r="V25" t="n">
-        <v>79.49299999999999</v>
+        <v>67.14700000000001</v>
       </c>
       <c r="W25" t="n">
-        <v>0.754</v>
+        <v>0.539</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B26" t="n">
-        <v>348.093</v>
+        <v>231.415</v>
       </c>
       <c r="C26" t="n">
-        <v>237.63</v>
+        <v>118.715</v>
       </c>
       <c r="D26" t="n">
-        <v>45.878</v>
+        <v>45.53</v>
       </c>
       <c r="E26" t="n">
-        <v>530.1319999999999</v>
+        <v>122.945</v>
       </c>
       <c r="F26" t="n">
-        <v>75.474</v>
+        <v>45.213</v>
       </c>
       <c r="G26" t="n">
-        <v>58.164</v>
+        <v>53.138</v>
       </c>
       <c r="H26" t="n">
-        <v>85.092</v>
+        <v>71.97</v>
       </c>
       <c r="I26" t="n">
         <v>4.46</v>
       </c>
       <c r="J26" t="n">
-        <v>3.666</v>
+        <v>3.242</v>
       </c>
       <c r="K26" t="n">
-        <v>300.409</v>
+        <v>32.838</v>
       </c>
       <c r="L26" t="n">
-        <v>261.507</v>
+        <v>250.054</v>
       </c>
       <c r="M26" t="n">
         <v>0</v>
       </c>
       <c r="N26" t="n">
-        <v>3.923</v>
+        <v>2.864</v>
       </c>
       <c r="O26" t="n">
         <v>0</v>
@@ -2834,224 +2770,1934 @@
         <v>0</v>
       </c>
       <c r="S26" t="n">
-        <v>0.645</v>
+        <v>0</v>
       </c>
       <c r="T26" t="n">
         <v>6.022</v>
       </c>
       <c r="U26" t="n">
-        <v>0.754</v>
+        <v>0.539</v>
       </c>
       <c r="V26" t="n">
-        <v>85.092</v>
+        <v>71.97</v>
       </c>
       <c r="W26" t="n">
-        <v>0.754</v>
+        <v>0.539</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B27" t="n">
-        <v>358.168</v>
+        <v>239.3</v>
       </c>
       <c r="C27" t="n">
-        <v>374.324</v>
+        <v>185.902</v>
       </c>
       <c r="D27" t="n">
-        <v>45.878</v>
+        <v>45.53</v>
       </c>
       <c r="E27" t="n">
-        <v>568.165</v>
+        <v>122.945</v>
       </c>
       <c r="F27" t="n">
-        <v>82.17100000000001</v>
+        <v>45.213</v>
       </c>
       <c r="G27" t="n">
-        <v>58.164</v>
+        <v>57.829</v>
       </c>
       <c r="H27" t="n">
-        <v>87.72799999999999</v>
+        <v>77.569</v>
       </c>
       <c r="I27" t="n">
         <v>4.46</v>
       </c>
       <c r="J27" t="n">
+        <v>3.242</v>
+      </c>
+      <c r="K27" t="n">
+        <v>32.838</v>
+      </c>
+      <c r="L27" t="n">
+        <v>251.097</v>
+      </c>
+      <c r="M27" t="n">
+        <v>0</v>
+      </c>
+      <c r="N27" t="n">
+        <v>2.864</v>
+      </c>
+      <c r="O27" t="n">
+        <v>0</v>
+      </c>
+      <c r="P27" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q27" t="n">
+        <v>0.14</v>
+      </c>
+      <c r="R27" t="n">
+        <v>0</v>
+      </c>
+      <c r="S27" t="n">
+        <v>0</v>
+      </c>
+      <c r="T27" t="n">
+        <v>6.022</v>
+      </c>
+      <c r="U27" t="n">
+        <v>0.539</v>
+      </c>
+      <c r="V27" t="n">
+        <v>77.569</v>
+      </c>
+      <c r="W27" t="n">
+        <v>0.539</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>21</v>
+      </c>
+      <c r="B28" t="n">
+        <v>245.289</v>
+      </c>
+      <c r="C28" t="n">
+        <v>317.429</v>
+      </c>
+      <c r="D28" t="n">
+        <v>45.53</v>
+      </c>
+      <c r="E28" t="n">
+        <v>137.64</v>
+      </c>
+      <c r="F28" t="n">
+        <v>51.909</v>
+      </c>
+      <c r="G28" t="n">
+        <v>57.829</v>
+      </c>
+      <c r="H28" t="n">
+        <v>80.205</v>
+      </c>
+      <c r="I28" t="n">
+        <v>4.46</v>
+      </c>
+      <c r="J28" t="n">
+        <v>3.242</v>
+      </c>
+      <c r="K28" t="n">
+        <v>35.309</v>
+      </c>
+      <c r="L28" t="n">
+        <v>251.325</v>
+      </c>
+      <c r="M28" t="n">
+        <v>0</v>
+      </c>
+      <c r="N28" t="n">
+        <v>2.864</v>
+      </c>
+      <c r="O28" t="n">
+        <v>0</v>
+      </c>
+      <c r="P28" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q28" t="n">
+        <v>0.14</v>
+      </c>
+      <c r="R28" t="n">
+        <v>0</v>
+      </c>
+      <c r="S28" t="n">
+        <v>0</v>
+      </c>
+      <c r="T28" t="n">
+        <v>6.949</v>
+      </c>
+      <c r="U28" t="n">
+        <v>0.539</v>
+      </c>
+      <c r="V28" t="n">
+        <v>80.205</v>
+      </c>
+      <c r="W28" t="n">
+        <v>0.539</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="1" t="inlineStr">
+        <is>
+          <t>BLOCK 2 — ALL seizures (convulsive + non-convulsive)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>X  (day)</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>EGFP 25</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>EGFP 31</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>EGFP 33</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>EGFP 355675</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>EGFP 355679</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="inlineStr">
+        <is>
+          <t>EGFP 372833</t>
+        </is>
+      </c>
+      <c r="H31" s="2" t="inlineStr">
+        <is>
+          <t>EGFP 372838</t>
+        </is>
+      </c>
+      <c r="I31" s="2" t="inlineStr">
+        <is>
+          <t>SV2A 24</t>
+        </is>
+      </c>
+      <c r="J31" s="2" t="inlineStr">
+        <is>
+          <t>SV2A 26</t>
+        </is>
+      </c>
+      <c r="K31" s="2" t="inlineStr">
+        <is>
+          <t>SV2A 29</t>
+        </is>
+      </c>
+      <c r="L31" s="2" t="inlineStr">
+        <is>
+          <t>SV2A 32</t>
+        </is>
+      </c>
+      <c r="M31" s="2" t="inlineStr">
+        <is>
+          <t>SV2A 355668</t>
+        </is>
+      </c>
+      <c r="N31" s="2" t="inlineStr">
+        <is>
+          <t>SV2A 355669</t>
+        </is>
+      </c>
+      <c r="O31" s="2" t="inlineStr">
+        <is>
+          <t>SV2A 355670</t>
+        </is>
+      </c>
+      <c r="P31" s="2" t="inlineStr">
+        <is>
+          <t>SV2A 355673</t>
+        </is>
+      </c>
+      <c r="Q31" s="2" t="inlineStr">
+        <is>
+          <t>SV2A 355677</t>
+        </is>
+      </c>
+      <c r="R31" s="2" t="inlineStr">
+        <is>
+          <t>SV2A 372828</t>
+        </is>
+      </c>
+      <c r="S31" s="2" t="inlineStr">
+        <is>
+          <t>SV2A 372829</t>
+        </is>
+      </c>
+      <c r="T31" s="2" t="inlineStr">
+        <is>
+          <t>SV2A 372830</t>
+        </is>
+      </c>
+      <c r="U31" s="2" t="inlineStr">
+        <is>
+          <t>SV2A 372832</t>
+        </is>
+      </c>
+      <c r="V31" s="2" t="inlineStr">
+        <is>
+          <t>EGFP median</t>
+        </is>
+      </c>
+      <c r="W31" s="2" t="inlineStr">
+        <is>
+          <t>SV2A median</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>1</v>
+      </c>
+      <c r="B32" t="n">
+        <v>3.777</v>
+      </c>
+      <c r="C32" t="n">
+        <v>0</v>
+      </c>
+      <c r="D32" t="n">
+        <v>0</v>
+      </c>
+      <c r="E32" t="n">
+        <v>8.137</v>
+      </c>
+      <c r="F32" t="n">
+        <v>4.501</v>
+      </c>
+      <c r="G32" t="n">
+        <v>0</v>
+      </c>
+      <c r="H32" t="n">
+        <v>0</v>
+      </c>
+      <c r="I32" t="n">
+        <v>0</v>
+      </c>
+      <c r="J32" t="n">
+        <v>1.174</v>
+      </c>
+      <c r="K32" t="n">
+        <v>17.018</v>
+      </c>
+      <c r="L32" t="n">
+        <v>2.981</v>
+      </c>
+      <c r="M32" t="n">
+        <v>0</v>
+      </c>
+      <c r="N32" t="n">
+        <v>0</v>
+      </c>
+      <c r="O32" t="n">
+        <v>0</v>
+      </c>
+      <c r="P32" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q32" t="n">
+        <v>0</v>
+      </c>
+      <c r="R32" t="n">
+        <v>0</v>
+      </c>
+      <c r="S32" t="n">
+        <v>0</v>
+      </c>
+      <c r="T32" t="n">
+        <v>0</v>
+      </c>
+      <c r="U32" t="n">
+        <v>0</v>
+      </c>
+      <c r="V32" t="n">
+        <v>0</v>
+      </c>
+      <c r="W32" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>2</v>
+      </c>
+      <c r="B33" t="n">
+        <v>5.25</v>
+      </c>
+      <c r="C33" t="n">
+        <v>0</v>
+      </c>
+      <c r="D33" t="n">
+        <v>0</v>
+      </c>
+      <c r="E33" t="n">
+        <v>23.419</v>
+      </c>
+      <c r="F33" t="n">
+        <v>7.226</v>
+      </c>
+      <c r="G33" t="n">
+        <v>1.865</v>
+      </c>
+      <c r="H33" t="n">
+        <v>8.156000000000001</v>
+      </c>
+      <c r="I33" t="n">
+        <v>0</v>
+      </c>
+      <c r="J33" t="n">
+        <v>1.278</v>
+      </c>
+      <c r="K33" t="n">
+        <v>22.114</v>
+      </c>
+      <c r="L33" t="n">
+        <v>5.109</v>
+      </c>
+      <c r="M33" t="n">
+        <v>0</v>
+      </c>
+      <c r="N33" t="n">
+        <v>0</v>
+      </c>
+      <c r="O33" t="n">
+        <v>0</v>
+      </c>
+      <c r="P33" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q33" t="n">
+        <v>0</v>
+      </c>
+      <c r="R33" t="n">
+        <v>0</v>
+      </c>
+      <c r="S33" t="n">
+        <v>0</v>
+      </c>
+      <c r="T33" t="n">
+        <v>0</v>
+      </c>
+      <c r="U33" t="n">
+        <v>0</v>
+      </c>
+      <c r="V33" t="n">
+        <v>5.25</v>
+      </c>
+      <c r="W33" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>3</v>
+      </c>
+      <c r="B34" t="n">
+        <v>6.235</v>
+      </c>
+      <c r="C34" t="n">
+        <v>0</v>
+      </c>
+      <c r="D34" t="n">
+        <v>0</v>
+      </c>
+      <c r="E34" t="n">
+        <v>41.704</v>
+      </c>
+      <c r="F34" t="n">
+        <v>11.329</v>
+      </c>
+      <c r="G34" t="n">
+        <v>3.768</v>
+      </c>
+      <c r="H34" t="n">
+        <v>10.328</v>
+      </c>
+      <c r="I34" t="n">
+        <v>0</v>
+      </c>
+      <c r="J34" t="n">
+        <v>1.278</v>
+      </c>
+      <c r="K34" t="n">
+        <v>30.063</v>
+      </c>
+      <c r="L34" t="n">
+        <v>9.436999999999999</v>
+      </c>
+      <c r="M34" t="n">
+        <v>0</v>
+      </c>
+      <c r="N34" t="n">
+        <v>0.261</v>
+      </c>
+      <c r="O34" t="n">
+        <v>0</v>
+      </c>
+      <c r="P34" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q34" t="n">
+        <v>0</v>
+      </c>
+      <c r="R34" t="n">
+        <v>0</v>
+      </c>
+      <c r="S34" t="n">
+        <v>0.436</v>
+      </c>
+      <c r="T34" t="n">
+        <v>0.626</v>
+      </c>
+      <c r="U34" t="n">
+        <v>0</v>
+      </c>
+      <c r="V34" t="n">
+        <v>6.235</v>
+      </c>
+      <c r="W34" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>4</v>
+      </c>
+      <c r="B35" t="n">
+        <v>9.663</v>
+      </c>
+      <c r="C35" t="n">
+        <v>2.561</v>
+      </c>
+      <c r="D35" t="n">
+        <v>0</v>
+      </c>
+      <c r="E35" t="n">
+        <v>61.922</v>
+      </c>
+      <c r="F35" t="n">
+        <v>18.563</v>
+      </c>
+      <c r="G35" t="n">
+        <v>6.413</v>
+      </c>
+      <c r="H35" t="n">
+        <v>13.633</v>
+      </c>
+      <c r="I35" t="n">
+        <v>1.317</v>
+      </c>
+      <c r="J35" t="n">
+        <v>1.598</v>
+      </c>
+      <c r="K35" t="n">
+        <v>37.563</v>
+      </c>
+      <c r="L35" t="n">
+        <v>18.395</v>
+      </c>
+      <c r="M35" t="n">
+        <v>0</v>
+      </c>
+      <c r="N35" t="n">
+        <v>0.261</v>
+      </c>
+      <c r="O35" t="n">
+        <v>0</v>
+      </c>
+      <c r="P35" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q35" t="n">
+        <v>0</v>
+      </c>
+      <c r="R35" t="n">
+        <v>0</v>
+      </c>
+      <c r="S35" t="n">
+        <v>0.645</v>
+      </c>
+      <c r="T35" t="n">
+        <v>0.626</v>
+      </c>
+      <c r="U35" t="n">
+        <v>0</v>
+      </c>
+      <c r="V35" t="n">
+        <v>9.663</v>
+      </c>
+      <c r="W35" t="n">
+        <v>0.261</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>5</v>
+      </c>
+      <c r="B36" t="n">
+        <v>13.277</v>
+      </c>
+      <c r="C36" t="n">
+        <v>3.493</v>
+      </c>
+      <c r="D36" t="n">
+        <v>0</v>
+      </c>
+      <c r="E36" t="n">
+        <v>107.61</v>
+      </c>
+      <c r="F36" t="n">
+        <v>30.952</v>
+      </c>
+      <c r="G36" t="n">
+        <v>10.624</v>
+      </c>
+      <c r="H36" t="n">
+        <v>31.862</v>
+      </c>
+      <c r="I36" t="n">
+        <v>1.317</v>
+      </c>
+      <c r="J36" t="n">
+        <v>1.598</v>
+      </c>
+      <c r="K36" t="n">
+        <v>40.302</v>
+      </c>
+      <c r="L36" t="n">
+        <v>25.484</v>
+      </c>
+      <c r="M36" t="n">
+        <v>0</v>
+      </c>
+      <c r="N36" t="n">
+        <v>0.779</v>
+      </c>
+      <c r="O36" t="n">
+        <v>0</v>
+      </c>
+      <c r="P36" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q36" t="n">
+        <v>0</v>
+      </c>
+      <c r="R36" t="n">
+        <v>0</v>
+      </c>
+      <c r="S36" t="n">
+        <v>0.645</v>
+      </c>
+      <c r="T36" t="n">
+        <v>0.626</v>
+      </c>
+      <c r="U36" t="n">
+        <v>0</v>
+      </c>
+      <c r="V36" t="n">
+        <v>13.277</v>
+      </c>
+      <c r="W36" t="n">
+        <v>0.626</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>6</v>
+      </c>
+      <c r="B37" t="n">
+        <v>18.357</v>
+      </c>
+      <c r="C37" t="n">
+        <v>6.629</v>
+      </c>
+      <c r="D37" t="n">
+        <v>0</v>
+      </c>
+      <c r="E37" t="n">
+        <v>107.61</v>
+      </c>
+      <c r="F37" t="n">
+        <v>30.952</v>
+      </c>
+      <c r="G37" t="n">
+        <v>10.624</v>
+      </c>
+      <c r="H37" t="n">
+        <v>31.862</v>
+      </c>
+      <c r="I37" t="n">
+        <v>1.317</v>
+      </c>
+      <c r="J37" t="n">
+        <v>1.598</v>
+      </c>
+      <c r="K37" t="n">
+        <v>45.075</v>
+      </c>
+      <c r="L37" t="n">
+        <v>45.433</v>
+      </c>
+      <c r="M37" t="n">
+        <v>0</v>
+      </c>
+      <c r="N37" t="n">
+        <v>0.779</v>
+      </c>
+      <c r="O37" t="n">
+        <v>0</v>
+      </c>
+      <c r="P37" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q37" t="n">
+        <v>0</v>
+      </c>
+      <c r="R37" t="n">
+        <v>0</v>
+      </c>
+      <c r="S37" t="n">
+        <v>0.645</v>
+      </c>
+      <c r="T37" t="n">
+        <v>0.626</v>
+      </c>
+      <c r="U37" t="n">
+        <v>0</v>
+      </c>
+      <c r="V37" t="n">
+        <v>18.357</v>
+      </c>
+      <c r="W37" t="n">
+        <v>0.626</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>7</v>
+      </c>
+      <c r="B38" t="n">
+        <v>22.407</v>
+      </c>
+      <c r="C38" t="n">
+        <v>9.331</v>
+      </c>
+      <c r="D38" t="n">
+        <v>0</v>
+      </c>
+      <c r="E38" t="n">
+        <v>126.484</v>
+      </c>
+      <c r="F38" t="n">
+        <v>33.083</v>
+      </c>
+      <c r="G38" t="n">
+        <v>14.536</v>
+      </c>
+      <c r="H38" t="n">
+        <v>36.628</v>
+      </c>
+      <c r="I38" t="n">
+        <v>1.317</v>
+      </c>
+      <c r="J38" t="n">
+        <v>1.598</v>
+      </c>
+      <c r="K38" t="n">
+        <v>67.09999999999999</v>
+      </c>
+      <c r="L38" t="n">
+        <v>63.464</v>
+      </c>
+      <c r="M38" t="n">
+        <v>0</v>
+      </c>
+      <c r="N38" t="n">
+        <v>0.779</v>
+      </c>
+      <c r="O38" t="n">
+        <v>0</v>
+      </c>
+      <c r="P38" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q38" t="n">
+        <v>0</v>
+      </c>
+      <c r="R38" t="n">
+        <v>0</v>
+      </c>
+      <c r="S38" t="n">
+        <v>0.645</v>
+      </c>
+      <c r="T38" t="n">
+        <v>1.276</v>
+      </c>
+      <c r="U38" t="n">
+        <v>0</v>
+      </c>
+      <c r="V38" t="n">
+        <v>22.407</v>
+      </c>
+      <c r="W38" t="n">
+        <v>0.645</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>8</v>
+      </c>
+      <c r="B39" t="n">
+        <v>28.332</v>
+      </c>
+      <c r="C39" t="n">
+        <v>13.248</v>
+      </c>
+      <c r="D39" t="n">
+        <v>0</v>
+      </c>
+      <c r="E39" t="n">
+        <v>158.689</v>
+      </c>
+      <c r="F39" t="n">
+        <v>40.131</v>
+      </c>
+      <c r="G39" t="n">
+        <v>18.88</v>
+      </c>
+      <c r="H39" t="n">
+        <v>36.628</v>
+      </c>
+      <c r="I39" t="n">
+        <v>1.317</v>
+      </c>
+      <c r="J39" t="n">
+        <v>1.598</v>
+      </c>
+      <c r="K39" t="n">
+        <v>111.623</v>
+      </c>
+      <c r="L39" t="n">
+        <v>81.935</v>
+      </c>
+      <c r="M39" t="n">
+        <v>0</v>
+      </c>
+      <c r="N39" t="n">
+        <v>0.889</v>
+      </c>
+      <c r="O39" t="n">
+        <v>0</v>
+      </c>
+      <c r="P39" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q39" t="n">
+        <v>0</v>
+      </c>
+      <c r="R39" t="n">
+        <v>0</v>
+      </c>
+      <c r="S39" t="n">
+        <v>0.645</v>
+      </c>
+      <c r="T39" t="n">
+        <v>2.044</v>
+      </c>
+      <c r="U39" t="n">
+        <v>0</v>
+      </c>
+      <c r="V39" t="n">
+        <v>28.332</v>
+      </c>
+      <c r="W39" t="n">
+        <v>0.645</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>9</v>
+      </c>
+      <c r="B40" t="n">
+        <v>33.647</v>
+      </c>
+      <c r="C40" t="n">
+        <v>18.568</v>
+      </c>
+      <c r="D40" t="n">
+        <v>0.256</v>
+      </c>
+      <c r="E40" t="n">
+        <v>194.037</v>
+      </c>
+      <c r="F40" t="n">
+        <v>44.558</v>
+      </c>
+      <c r="G40" t="n">
+        <v>20.52</v>
+      </c>
+      <c r="H40" t="n">
+        <v>37.625</v>
+      </c>
+      <c r="I40" t="n">
+        <v>1.317</v>
+      </c>
+      <c r="J40" t="n">
+        <v>1.598</v>
+      </c>
+      <c r="K40" t="n">
+        <v>144.082</v>
+      </c>
+      <c r="L40" t="n">
+        <v>103.187</v>
+      </c>
+      <c r="M40" t="n">
+        <v>0</v>
+      </c>
+      <c r="N40" t="n">
+        <v>0.889</v>
+      </c>
+      <c r="O40" t="n">
+        <v>0</v>
+      </c>
+      <c r="P40" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q40" t="n">
+        <v>0</v>
+      </c>
+      <c r="R40" t="n">
+        <v>0</v>
+      </c>
+      <c r="S40" t="n">
+        <v>0.645</v>
+      </c>
+      <c r="T40" t="n">
+        <v>2.044</v>
+      </c>
+      <c r="U40" t="n">
+        <v>0</v>
+      </c>
+      <c r="V40" t="n">
+        <v>33.647</v>
+      </c>
+      <c r="W40" t="n">
+        <v>0.645</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>10</v>
+      </c>
+      <c r="B41" t="n">
+        <v>42.312</v>
+      </c>
+      <c r="C41" t="n">
+        <v>24.996</v>
+      </c>
+      <c r="D41" t="n">
+        <v>0.756</v>
+      </c>
+      <c r="E41" t="n">
+        <v>251.443</v>
+      </c>
+      <c r="F41" t="n">
+        <v>46.512</v>
+      </c>
+      <c r="G41" t="n">
+        <v>22.846</v>
+      </c>
+      <c r="H41" t="n">
+        <v>46.251</v>
+      </c>
+      <c r="I41" t="n">
+        <v>2.835</v>
+      </c>
+      <c r="J41" t="n">
+        <v>1.598</v>
+      </c>
+      <c r="K41" t="n">
+        <v>160.912</v>
+      </c>
+      <c r="L41" t="n">
+        <v>119.698</v>
+      </c>
+      <c r="M41" t="n">
+        <v>0</v>
+      </c>
+      <c r="N41" t="n">
+        <v>1.704</v>
+      </c>
+      <c r="O41" t="n">
+        <v>0</v>
+      </c>
+      <c r="P41" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q41" t="n">
+        <v>0</v>
+      </c>
+      <c r="R41" t="n">
+        <v>0</v>
+      </c>
+      <c r="S41" t="n">
+        <v>0.645</v>
+      </c>
+      <c r="T41" t="n">
+        <v>2.488</v>
+      </c>
+      <c r="U41" t="n">
+        <v>0</v>
+      </c>
+      <c r="V41" t="n">
+        <v>42.312</v>
+      </c>
+      <c r="W41" t="n">
+        <v>0.645</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>11</v>
+      </c>
+      <c r="B42" t="n">
+        <v>60.44</v>
+      </c>
+      <c r="C42" t="n">
+        <v>35.622</v>
+      </c>
+      <c r="D42" t="n">
+        <v>4.661</v>
+      </c>
+      <c r="E42" t="n">
+        <v>251.443</v>
+      </c>
+      <c r="F42" t="n">
+        <v>46.512</v>
+      </c>
+      <c r="G42" t="n">
+        <v>27.772</v>
+      </c>
+      <c r="H42" t="n">
+        <v>51.071</v>
+      </c>
+      <c r="I42" t="n">
+        <v>3.798</v>
+      </c>
+      <c r="J42" t="n">
+        <v>3.046</v>
+      </c>
+      <c r="K42" t="n">
+        <v>189.689</v>
+      </c>
+      <c r="L42" t="n">
+        <v>151.666</v>
+      </c>
+      <c r="M42" t="n">
+        <v>0</v>
+      </c>
+      <c r="N42" t="n">
+        <v>1.704</v>
+      </c>
+      <c r="O42" t="n">
+        <v>0</v>
+      </c>
+      <c r="P42" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q42" t="n">
+        <v>0</v>
+      </c>
+      <c r="R42" t="n">
+        <v>0</v>
+      </c>
+      <c r="S42" t="n">
+        <v>0.645</v>
+      </c>
+      <c r="T42" t="n">
+        <v>2.488</v>
+      </c>
+      <c r="U42" t="n">
+        <v>0</v>
+      </c>
+      <c r="V42" t="n">
+        <v>46.512</v>
+      </c>
+      <c r="W42" t="n">
+        <v>0.645</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>12</v>
+      </c>
+      <c r="B43" t="n">
+        <v>67.619</v>
+      </c>
+      <c r="C43" t="n">
+        <v>40.11</v>
+      </c>
+      <c r="D43" t="n">
+        <v>9.643000000000001</v>
+      </c>
+      <c r="E43" t="n">
+        <v>280.865</v>
+      </c>
+      <c r="F43" t="n">
+        <v>52.65</v>
+      </c>
+      <c r="G43" t="n">
+        <v>37.209</v>
+      </c>
+      <c r="H43" t="n">
+        <v>58.696</v>
+      </c>
+      <c r="I43" t="n">
+        <v>4.46</v>
+      </c>
+      <c r="J43" t="n">
         <v>3.666</v>
       </c>
-      <c r="K27" t="n">
+      <c r="K43" t="n">
+        <v>212.859</v>
+      </c>
+      <c r="L43" t="n">
+        <v>168.506</v>
+      </c>
+      <c r="M43" t="n">
+        <v>0</v>
+      </c>
+      <c r="N43" t="n">
+        <v>1.704</v>
+      </c>
+      <c r="O43" t="n">
+        <v>0</v>
+      </c>
+      <c r="P43" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q43" t="n">
+        <v>0</v>
+      </c>
+      <c r="R43" t="n">
+        <v>0</v>
+      </c>
+      <c r="S43" t="n">
+        <v>0.645</v>
+      </c>
+      <c r="T43" t="n">
+        <v>3.557</v>
+      </c>
+      <c r="U43" t="n">
+        <v>0</v>
+      </c>
+      <c r="V43" t="n">
+        <v>52.65</v>
+      </c>
+      <c r="W43" t="n">
+        <v>0.645</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="n">
+        <v>13</v>
+      </c>
+      <c r="B44" t="n">
+        <v>80.44799999999999</v>
+      </c>
+      <c r="C44" t="n">
+        <v>46.453</v>
+      </c>
+      <c r="D44" t="n">
+        <v>16.988</v>
+      </c>
+      <c r="E44" t="n">
+        <v>323.538</v>
+      </c>
+      <c r="F44" t="n">
+        <v>57.78</v>
+      </c>
+      <c r="G44" t="n">
+        <v>37.209</v>
+      </c>
+      <c r="H44" t="n">
+        <v>58.696</v>
+      </c>
+      <c r="I44" t="n">
+        <v>4.46</v>
+      </c>
+      <c r="J44" t="n">
+        <v>3.666</v>
+      </c>
+      <c r="K44" t="n">
+        <v>230.531</v>
+      </c>
+      <c r="L44" t="n">
+        <v>187.336</v>
+      </c>
+      <c r="M44" t="n">
+        <v>0</v>
+      </c>
+      <c r="N44" t="n">
+        <v>2.314</v>
+      </c>
+      <c r="O44" t="n">
+        <v>0</v>
+      </c>
+      <c r="P44" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q44" t="n">
+        <v>0</v>
+      </c>
+      <c r="R44" t="n">
+        <v>0</v>
+      </c>
+      <c r="S44" t="n">
+        <v>0.645</v>
+      </c>
+      <c r="T44" t="n">
+        <v>3.557</v>
+      </c>
+      <c r="U44" t="n">
+        <v>0</v>
+      </c>
+      <c r="V44" t="n">
+        <v>57.78</v>
+      </c>
+      <c r="W44" t="n">
+        <v>0.645</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="n">
+        <v>14</v>
+      </c>
+      <c r="B45" t="n">
+        <v>90.556</v>
+      </c>
+      <c r="C45" t="n">
+        <v>52.48</v>
+      </c>
+      <c r="D45" t="n">
+        <v>22.657</v>
+      </c>
+      <c r="E45" t="n">
+        <v>323.538</v>
+      </c>
+      <c r="F45" t="n">
+        <v>57.78</v>
+      </c>
+      <c r="G45" t="n">
+        <v>40.414</v>
+      </c>
+      <c r="H45" t="n">
+        <v>61.623</v>
+      </c>
+      <c r="I45" t="n">
+        <v>4.46</v>
+      </c>
+      <c r="J45" t="n">
+        <v>3.666</v>
+      </c>
+      <c r="K45" t="n">
+        <v>269.418</v>
+      </c>
+      <c r="L45" t="n">
+        <v>201.509</v>
+      </c>
+      <c r="M45" t="n">
+        <v>0</v>
+      </c>
+      <c r="N45" t="n">
+        <v>2.314</v>
+      </c>
+      <c r="O45" t="n">
+        <v>0</v>
+      </c>
+      <c r="P45" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q45" t="n">
+        <v>0</v>
+      </c>
+      <c r="R45" t="n">
+        <v>0</v>
+      </c>
+      <c r="S45" t="n">
+        <v>0.645</v>
+      </c>
+      <c r="T45" t="n">
+        <v>3.557</v>
+      </c>
+      <c r="U45" t="n">
+        <v>0</v>
+      </c>
+      <c r="V45" t="n">
+        <v>57.78</v>
+      </c>
+      <c r="W45" t="n">
+        <v>0.645</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="n">
+        <v>15</v>
+      </c>
+      <c r="B46" t="n">
+        <v>123.142</v>
+      </c>
+      <c r="C46" t="n">
+        <v>65.702</v>
+      </c>
+      <c r="D46" t="n">
+        <v>31.719</v>
+      </c>
+      <c r="E46" t="n">
+        <v>351.599</v>
+      </c>
+      <c r="F46" t="n">
+        <v>60.956</v>
+      </c>
+      <c r="G46" t="n">
+        <v>44.871</v>
+      </c>
+      <c r="H46" t="n">
+        <v>64.04600000000001</v>
+      </c>
+      <c r="I46" t="n">
+        <v>4.46</v>
+      </c>
+      <c r="J46" t="n">
+        <v>3.666</v>
+      </c>
+      <c r="K46" t="n">
+        <v>274.214</v>
+      </c>
+      <c r="L46" t="n">
+        <v>226.165</v>
+      </c>
+      <c r="M46" t="n">
+        <v>0</v>
+      </c>
+      <c r="N46" t="n">
+        <v>2.314</v>
+      </c>
+      <c r="O46" t="n">
+        <v>0</v>
+      </c>
+      <c r="P46" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q46" t="n">
+        <v>0</v>
+      </c>
+      <c r="R46" t="n">
+        <v>0</v>
+      </c>
+      <c r="S46" t="n">
+        <v>0.645</v>
+      </c>
+      <c r="T46" t="n">
+        <v>3.557</v>
+      </c>
+      <c r="U46" t="n">
+        <v>0</v>
+      </c>
+      <c r="V46" t="n">
+        <v>64.04600000000001</v>
+      </c>
+      <c r="W46" t="n">
+        <v>0.645</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="n">
+        <v>16</v>
+      </c>
+      <c r="B47" t="n">
+        <v>193.203</v>
+      </c>
+      <c r="C47" t="n">
+        <v>72.986</v>
+      </c>
+      <c r="D47" t="n">
+        <v>38.706</v>
+      </c>
+      <c r="E47" t="n">
+        <v>392.31</v>
+      </c>
+      <c r="F47" t="n">
+        <v>62.511</v>
+      </c>
+      <c r="G47" t="n">
+        <v>47.128</v>
+      </c>
+      <c r="H47" t="n">
+        <v>67.16800000000001</v>
+      </c>
+      <c r="I47" t="n">
+        <v>4.46</v>
+      </c>
+      <c r="J47" t="n">
+        <v>3.666</v>
+      </c>
+      <c r="K47" t="n">
+        <v>281.802</v>
+      </c>
+      <c r="L47" t="n">
+        <v>232.404</v>
+      </c>
+      <c r="M47" t="n">
+        <v>0</v>
+      </c>
+      <c r="N47" t="n">
+        <v>2.314</v>
+      </c>
+      <c r="O47" t="n">
+        <v>0</v>
+      </c>
+      <c r="P47" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q47" t="n">
+        <v>0</v>
+      </c>
+      <c r="R47" t="n">
+        <v>0</v>
+      </c>
+      <c r="S47" t="n">
+        <v>0.645</v>
+      </c>
+      <c r="T47" t="n">
+        <v>4.415</v>
+      </c>
+      <c r="U47" t="n">
+        <v>0.539</v>
+      </c>
+      <c r="V47" t="n">
+        <v>67.16800000000001</v>
+      </c>
+      <c r="W47" t="n">
+        <v>0.645</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="n">
+        <v>17</v>
+      </c>
+      <c r="B48" t="n">
+        <v>245.679</v>
+      </c>
+      <c r="C48" t="n">
+        <v>85.22499999999999</v>
+      </c>
+      <c r="D48" t="n">
+        <v>45.181</v>
+      </c>
+      <c r="E48" t="n">
+        <v>435.401</v>
+      </c>
+      <c r="F48" t="n">
+        <v>65.43600000000001</v>
+      </c>
+      <c r="G48" t="n">
+        <v>48.834</v>
+      </c>
+      <c r="H48" t="n">
+        <v>70.408</v>
+      </c>
+      <c r="I48" t="n">
+        <v>4.46</v>
+      </c>
+      <c r="J48" t="n">
+        <v>3.666</v>
+      </c>
+      <c r="K48" t="n">
+        <v>299.691</v>
+      </c>
+      <c r="L48" t="n">
+        <v>252.786</v>
+      </c>
+      <c r="M48" t="n">
+        <v>0</v>
+      </c>
+      <c r="N48" t="n">
+        <v>2.314</v>
+      </c>
+      <c r="O48" t="n">
+        <v>0</v>
+      </c>
+      <c r="P48" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q48" t="n">
+        <v>0</v>
+      </c>
+      <c r="R48" t="n">
+        <v>0</v>
+      </c>
+      <c r="S48" t="n">
+        <v>0.645</v>
+      </c>
+      <c r="T48" t="n">
+        <v>5.465</v>
+      </c>
+      <c r="U48" t="n">
+        <v>0.539</v>
+      </c>
+      <c r="V48" t="n">
+        <v>70.408</v>
+      </c>
+      <c r="W48" t="n">
+        <v>0.645</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="n">
+        <v>18</v>
+      </c>
+      <c r="B49" t="n">
+        <v>334.378</v>
+      </c>
+      <c r="C49" t="n">
+        <v>168.448</v>
+      </c>
+      <c r="D49" t="n">
+        <v>45.878</v>
+      </c>
+      <c r="E49" t="n">
+        <v>481.811</v>
+      </c>
+      <c r="F49" t="n">
+        <v>69.66800000000001</v>
+      </c>
+      <c r="G49" t="n">
+        <v>50.579</v>
+      </c>
+      <c r="H49" t="n">
+        <v>74.67</v>
+      </c>
+      <c r="I49" t="n">
+        <v>4.46</v>
+      </c>
+      <c r="J49" t="n">
+        <v>3.666</v>
+      </c>
+      <c r="K49" t="n">
+        <v>300.299</v>
+      </c>
+      <c r="L49" t="n">
+        <v>259.246</v>
+      </c>
+      <c r="M49" t="n">
+        <v>0</v>
+      </c>
+      <c r="N49" t="n">
+        <v>3.226</v>
+      </c>
+      <c r="O49" t="n">
+        <v>0</v>
+      </c>
+      <c r="P49" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q49" t="n">
+        <v>0</v>
+      </c>
+      <c r="R49" t="n">
+        <v>0</v>
+      </c>
+      <c r="S49" t="n">
+        <v>0.645</v>
+      </c>
+      <c r="T49" t="n">
+        <v>5.465</v>
+      </c>
+      <c r="U49" t="n">
+        <v>0.539</v>
+      </c>
+      <c r="V49" t="n">
+        <v>74.67</v>
+      </c>
+      <c r="W49" t="n">
+        <v>0.645</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="n">
+        <v>19</v>
+      </c>
+      <c r="B50" t="n">
+        <v>334.378</v>
+      </c>
+      <c r="C50" t="n">
+        <v>168.448</v>
+      </c>
+      <c r="D50" t="n">
+        <v>45.878</v>
+      </c>
+      <c r="E50" t="n">
+        <v>530.1319999999999</v>
+      </c>
+      <c r="F50" t="n">
+        <v>75.474</v>
+      </c>
+      <c r="G50" t="n">
+        <v>53.354</v>
+      </c>
+      <c r="H50" t="n">
+        <v>79.49299999999999</v>
+      </c>
+      <c r="I50" t="n">
+        <v>4.46</v>
+      </c>
+      <c r="J50" t="n">
+        <v>3.666</v>
+      </c>
+      <c r="K50" t="n">
+        <v>300.299</v>
+      </c>
+      <c r="L50" t="n">
+        <v>259.246</v>
+      </c>
+      <c r="M50" t="n">
+        <v>0</v>
+      </c>
+      <c r="N50" t="n">
+        <v>3.923</v>
+      </c>
+      <c r="O50" t="n">
+        <v>0</v>
+      </c>
+      <c r="P50" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q50" t="n">
+        <v>0.14</v>
+      </c>
+      <c r="R50" t="n">
+        <v>0</v>
+      </c>
+      <c r="S50" t="n">
+        <v>0.645</v>
+      </c>
+      <c r="T50" t="n">
+        <v>6.022</v>
+      </c>
+      <c r="U50" t="n">
+        <v>0.754</v>
+      </c>
+      <c r="V50" t="n">
+        <v>79.49299999999999</v>
+      </c>
+      <c r="W50" t="n">
+        <v>0.754</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="n">
+        <v>20</v>
+      </c>
+      <c r="B51" t="n">
+        <v>348.093</v>
+      </c>
+      <c r="C51" t="n">
+        <v>237.63</v>
+      </c>
+      <c r="D51" t="n">
+        <v>45.878</v>
+      </c>
+      <c r="E51" t="n">
+        <v>530.1319999999999</v>
+      </c>
+      <c r="F51" t="n">
+        <v>75.474</v>
+      </c>
+      <c r="G51" t="n">
+        <v>58.164</v>
+      </c>
+      <c r="H51" t="n">
+        <v>85.092</v>
+      </c>
+      <c r="I51" t="n">
+        <v>4.46</v>
+      </c>
+      <c r="J51" t="n">
+        <v>3.666</v>
+      </c>
+      <c r="K51" t="n">
+        <v>300.409</v>
+      </c>
+      <c r="L51" t="n">
+        <v>261.507</v>
+      </c>
+      <c r="M51" t="n">
+        <v>0</v>
+      </c>
+      <c r="N51" t="n">
+        <v>3.923</v>
+      </c>
+      <c r="O51" t="n">
+        <v>0</v>
+      </c>
+      <c r="P51" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q51" t="n">
+        <v>0.14</v>
+      </c>
+      <c r="R51" t="n">
+        <v>0</v>
+      </c>
+      <c r="S51" t="n">
+        <v>0.645</v>
+      </c>
+      <c r="T51" t="n">
+        <v>6.022</v>
+      </c>
+      <c r="U51" t="n">
+        <v>0.754</v>
+      </c>
+      <c r="V51" t="n">
+        <v>85.092</v>
+      </c>
+      <c r="W51" t="n">
+        <v>0.754</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="n">
+        <v>21</v>
+      </c>
+      <c r="B52" t="n">
+        <v>358.168</v>
+      </c>
+      <c r="C52" t="n">
+        <v>374.324</v>
+      </c>
+      <c r="D52" t="n">
+        <v>45.878</v>
+      </c>
+      <c r="E52" t="n">
+        <v>568.165</v>
+      </c>
+      <c r="F52" t="n">
+        <v>82.17100000000001</v>
+      </c>
+      <c r="G52" t="n">
+        <v>58.164</v>
+      </c>
+      <c r="H52" t="n">
+        <v>87.72799999999999</v>
+      </c>
+      <c r="I52" t="n">
+        <v>4.46</v>
+      </c>
+      <c r="J52" t="n">
+        <v>3.666</v>
+      </c>
+      <c r="K52" t="n">
         <v>303.729</v>
       </c>
-      <c r="L27" t="n">
+      <c r="L52" t="n">
         <v>262.823</v>
       </c>
-      <c r="M27" t="n">
-        <v>0</v>
-      </c>
-      <c r="N27" t="n">
+      <c r="M52" t="n">
+        <v>0</v>
+      </c>
+      <c r="N52" t="n">
         <v>3.923</v>
       </c>
-      <c r="O27" t="n">
-        <v>0</v>
-      </c>
-      <c r="P27" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q27" t="n">
+      <c r="O52" t="n">
+        <v>0</v>
+      </c>
+      <c r="P52" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q52" t="n">
         <v>0.439</v>
       </c>
-      <c r="R27" t="n">
-        <v>0</v>
-      </c>
-      <c r="S27" t="n">
+      <c r="R52" t="n">
+        <v>0</v>
+      </c>
+      <c r="S52" t="n">
         <v>0.645</v>
       </c>
-      <c r="T27" t="n">
+      <c r="T52" t="n">
         <v>6.949</v>
       </c>
-      <c r="U27" t="n">
+      <c r="U52" t="n">
         <v>0.754</v>
       </c>
-      <c r="V27" t="n">
+      <c r="V52" t="n">
         <v>87.72799999999999</v>
       </c>
-      <c r="W27" t="n">
+      <c r="W52" t="n">
         <v>0.754</v>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="1" t="inlineStr">
+    <row r="54">
+      <c r="A54" s="1" t="inlineStr">
         <is>
           <t>STATISTICS TO RUN IN PRISM</t>
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="3" t="inlineStr">
+    <row r="55">
+      <c r="A55" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">  The curves are descriptive. Test the ENDPOINT (day 21 total) only:</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="3" t="inlineStr">
+    <row r="56">
+      <c r="A56" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">  Analyze → Column analyses → t test (and nonparametric tests)</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="3" t="inlineStr">
+    <row r="57">
+      <c r="A57" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">         → 'Mann-Whitney test' (unpaired, two-tailed), EGFP vs SV2A.</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  EXPECTED: median EGFP 87.7 min, SV2A 0.8 min, p = 0.0032</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="3" t="inlineStr">
+    <row r="58">
+      <c r="A58" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  CONVULSIVE ONLY: median EGFP 80.2 min, SV2A 0.5 min, p = 0.0018</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ALL SEIZURES:    median EGFP 87.7 min, SV2A 0.8 min, p = 0.0032</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">  Do not run a 2-way ANOVA over days: cumulative values are not</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="3" t="inlineStr">
+    <row r="61">
+      <c r="A61" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">  independent across time, so the day factor is not interpretable.</t>
         </is>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" s="3" t="inlineStr"/>
-    </row>
-    <row r="37">
-      <c r="A37" s="3" t="inlineStr">
-        <is>
-          <t>PLOT MEDIAN, NOT MEAN +/- SEM. The SV2A group is bimodal — 4 animals</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="3" t="inlineStr">
-        <is>
-          <t>at exactly 0 for all 21 days and 2 non-responders as high as EGFP — so</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="3" t="inlineStr">
-        <is>
-          <t>the mean is dragged up and the error bars overlap (EGFP 225 +/- 78 vs</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="3" t="inlineStr">
-        <is>
-          <t>SV2A 45 +/- 29 min), which understates a difference the medians show</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="3" t="inlineStr">
-        <is>
-          <t>clearly (87.7 vs 0.8 min).</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="3" t="inlineStr"/>
-    </row>
-    <row r="43">
-      <c r="A43" s="3" t="inlineStr">
+    <row r="62">
+      <c r="A62" s="3" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="3" t="inlineStr">
+        <is>
+          <t>WHICH BLOCK: convulsive-only is recommended. Its 5/13 SV2A animals that</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="3" t="inlineStr">
+        <is>
+          <t>never seize are the SAME animals censored in the survival panel, so the</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="3" t="inlineStr">
+        <is>
+          <t>two panels cross-reference. All-seizures gives 4/13 at zero,</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="3" t="inlineStr">
+        <is>
+          <t>which a reader then has to reconcile against the survival panel.</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="3" t="inlineStr"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="3" t="inlineStr">
+        <is>
+          <t>PLOT MEDIAN, NOT MEAN +/- SEM. The SV2A group is bimodal — several</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="3" t="inlineStr">
+        <is>
+          <t>animals at exactly 0 for all 21 days and 2 non-responders as high as</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="3" t="inlineStr">
+        <is>
+          <t>EGFP — so the mean is dragged up and the error bars overlap, which</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="3" t="inlineStr">
+        <is>
+          <t>understates a difference the medians show clearly.</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="3" t="inlineStr"/>
+    </row>
+    <row r="73">
+      <c r="A73" s="3" t="inlineStr">
         <is>
           <t>ZEROS ARE REAL. A flat line along the axis means that animal never had</t>
         </is>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" s="3" t="inlineStr">
-        <is>
-          <t>a seizure; it is not a plotting floor. Use a LINEAR y-axis here — do not</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="3" t="inlineStr">
+    <row r="74">
+      <c r="A74" s="3" t="inlineStr">
+        <is>
+          <t>a seizure; it is not a plotting floor. Use a LINEAR y-axis — do not</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="3" t="inlineStr">
         <is>
           <t>log-transform, or the flat-at-zero animals cannot be drawn.</t>
         </is>
       </c>
     </row>
-    <row r="46">
-      <c r="A46" s="3" t="inlineStr"/>
-    </row>
-    <row r="47">
-      <c r="A47" s="3" t="inlineStr">
-        <is>
-          <t>NON-RESPONDERS: SV2A animals with the two highest totals are the two</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="3" t="inlineStr">
-        <is>
-          <t>climbing SV2A lines; naming them in the legend is worth doing, since the</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="3" t="inlineStr">
-        <is>
-          <t>responder/non-responder split is more informative than the group median.</t>
+    <row r="76">
+      <c r="A76" s="3" t="inlineStr"/>
+    </row>
+    <row r="77">
+      <c r="A77" s="3" t="inlineStr">
+        <is>
+          <t>Y-AXIS LABEL: 'Cumulative convulsive seizure time (min)' for block 1,</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="3" t="inlineStr">
+        <is>
+          <t>or 'Cumulative seizure time (min)' for block 2. State which in the legend.</t>
         </is>
       </c>
     </row>

</xml_diff>